<commit_message>
#16 Resistor added SMA Connector and Capacitor C6 Changed
</commit_message>
<xml_diff>
--- a/Design Files/LTE-Module-v2.0/BOM/Client_BOM_v2.0.xlsx
+++ b/Design Files/LTE-Module-v2.0/BOM/Client_BOM_v2.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="192">
   <si>
     <t>Component list</t>
   </si>
@@ -36,12 +36,6 @@
     <t>#</t>
   </si>
   <si>
-    <t>Bill of Materials for Project [LTE_MODULE_v2.0.PrjPcb] (No PCB Document Selected)</t>
-  </si>
-  <si>
-    <t>LTE_MODULE_v2.0.PrjPcb</t>
-  </si>
-  <si>
     <t>None</t>
   </si>
   <si>
@@ -168,9 +162,6 @@
     <t>R8, R11, R14, R18</t>
   </si>
   <si>
-    <t>R12, R15, R16</t>
-  </si>
-  <si>
     <t>U1</t>
   </si>
   <si>
@@ -201,9 +192,6 @@
     <t>CAP CER 0.1UF 50V X5R 0603</t>
   </si>
   <si>
-    <t>220uF 5.4mm 10V 6.3mm ±20% SMD,D6.3xL5.4mm Aluminum Electrolytic Capacitors - SMD ROHS</t>
-  </si>
-  <si>
     <t>CAP CER 1UF 25V X5R 0603</t>
   </si>
   <si>
@@ -228,9 +216,6 @@
     <t>6V 500mA 40A 1A 0603 Resettable Fuses ROHS</t>
   </si>
   <si>
-    <t>Sma Female Connector, Pcb Edge Mount Rohs Compliant: Yes</t>
-  </si>
-  <si>
     <t>PCI Express Mini Card (Mini PCIe)</t>
   </si>
   <si>
@@ -294,9 +279,6 @@
     <t>Cap-0402</t>
   </si>
   <si>
-    <t>RT1A221M0605</t>
-  </si>
-  <si>
     <t>cap-0402</t>
   </si>
   <si>
@@ -384,9 +366,6 @@
     <t>SMD0603-050</t>
   </si>
   <si>
-    <t>CON-SMA-EDGE-S</t>
-  </si>
-  <si>
     <t>POGO Connector 4 Pin</t>
   </si>
   <si>
@@ -447,9 +426,6 @@
     <t>Yageo</t>
   </si>
   <si>
-    <t>ROQANG</t>
-  </si>
-  <si>
     <t>TDK</t>
   </si>
   <si>
@@ -468,9 +444,6 @@
     <t>TECHFUSE</t>
   </si>
   <si>
-    <t>RF Solutions</t>
-  </si>
-  <si>
     <t>XKB Connectivity</t>
   </si>
   <si>
@@ -592,6 +565,36 @@
   </si>
   <si>
     <t>Custom Supplier</t>
+  </si>
+  <si>
+    <t>1 Inner bore SMA Board Edge Bend -55℃~+155℃ 50Ω Plugin RF Connectors / Coaxial Connectors ROHS</t>
+  </si>
+  <si>
+    <t>HJ-SMA508</t>
+  </si>
+  <si>
+    <t>HJ Tech</t>
+  </si>
+  <si>
+    <t>CAP TANT 220UF 20% 6.3V SMD</t>
+  </si>
+  <si>
+    <t>Case-B</t>
+  </si>
+  <si>
+    <t>TLJB227M006R0500</t>
+  </si>
+  <si>
+    <t>Kyocera AVX</t>
+  </si>
+  <si>
+    <t>R12, R15, R16, R19, R20</t>
+  </si>
+  <si>
+    <t>Bill of Materials for Project [LTE_MODULE_v2.0.]</t>
+  </si>
+  <si>
+    <t>LTE_MODULE_v2.0</t>
   </si>
 </sst>
 </file>
@@ -1571,9 +1574,9 @@
     <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
     <col min="6" max="6" width="26.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="33.42578125" customWidth="1"/>
-    <col min="9" max="9" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.5703125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="16.5703125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="18.28515625" bestFit="1" customWidth="1"/>
@@ -1610,11 +1613,11 @@
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="51" t="s">
-        <v>5</v>
+        <v>190</v>
       </c>
       <c r="G2" s="11"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="11"/>
       <c r="J2" s="3"/>
       <c r="K2" s="3"/>
       <c r="L2" s="3"/>
@@ -1632,11 +1635,11 @@
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="52" t="s">
-        <v>6</v>
+        <v>191</v>
       </c>
       <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="12"/>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
@@ -1654,11 +1657,11 @@
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="53" t="s">
-        <v>6</v>
+        <v>191</v>
       </c>
       <c r="G4" s="13"/>
-      <c r="H4" s="13"/>
-      <c r="I4" s="6"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="13"/>
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
       <c r="L4" s="6"/>
@@ -1676,11 +1679,11 @@
       </c>
       <c r="E5" s="12"/>
       <c r="F5" s="54" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G5" s="14"/>
-      <c r="H5" s="14"/>
-      <c r="I5" s="5"/>
+      <c r="H5" s="5"/>
+      <c r="I5" s="14"/>
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
       <c r="L5" s="5"/>
@@ -1697,8 +1700,8 @@
       <c r="E6" s="15"/>
       <c r="F6" s="16"/>
       <c r="G6" s="14"/>
-      <c r="H6" s="14"/>
-      <c r="I6" s="5"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="14"/>
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
       <c r="L6" s="5"/>
@@ -1715,8 +1718,8 @@
       <c r="E7" s="17"/>
       <c r="F7" s="18"/>
       <c r="G7" s="17"/>
-      <c r="H7" s="17"/>
-      <c r="I7" s="7"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="17"/>
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
       <c r="L7" s="7"/>
@@ -1733,8 +1736,8 @@
       <c r="E8" s="27"/>
       <c r="F8" s="28"/>
       <c r="G8" s="17"/>
-      <c r="H8" s="17"/>
-      <c r="I8" s="7"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="17"/>
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
       <c r="L8" s="7"/>
@@ -1749,46 +1752,46 @@
         <v>4</v>
       </c>
       <c r="C9" s="29" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D9" s="29" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E9" s="30" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F9" s="29" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="G9" s="30" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="H9" s="29" t="s">
+        <v>130</v>
+      </c>
+      <c r="I9" s="29" t="s">
+        <v>165</v>
+      </c>
+      <c r="J9" s="29" t="s">
+        <v>167</v>
+      </c>
+      <c r="K9" s="29" t="s">
+        <v>164</v>
+      </c>
+      <c r="L9" s="29" t="s">
+        <v>166</v>
+      </c>
+      <c r="M9" s="29" t="s">
+        <v>172</v>
+      </c>
+      <c r="N9" s="29" t="s">
         <v>174</v>
       </c>
-      <c r="I9" s="29" t="s">
-        <v>137</v>
-      </c>
-      <c r="J9" s="29" t="s">
-        <v>176</v>
-      </c>
-      <c r="K9" s="29" t="s">
-        <v>173</v>
-      </c>
-      <c r="L9" s="29" t="s">
+      <c r="O9" s="29" t="s">
         <v>175</v>
       </c>
-      <c r="M9" s="29" t="s">
-        <v>181</v>
-      </c>
-      <c r="N9" s="29" t="s">
-        <v>183</v>
-      </c>
-      <c r="O9" s="29" t="s">
-        <v>184</v>
-      </c>
       <c r="P9" s="29" t="s">
-        <v>180</v>
+        <v>171</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1798,28 +1801,28 @@
         <v>1</v>
       </c>
       <c r="C10" s="56" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D10" s="36" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E10" s="37" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F10" s="36" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="G10" s="37" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="H10" s="36" t="s">
-        <v>177</v>
+        <v>131</v>
       </c>
       <c r="I10" s="36" t="s">
-        <v>138</v>
+        <v>168</v>
       </c>
       <c r="J10" s="36" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="K10" s="36">
         <v>1</v>
@@ -1829,7 +1832,7 @@
         <v>5</v>
       </c>
       <c r="M10" s="59" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="N10" s="61">
         <v>0.9</v>
@@ -1847,26 +1850,28 @@
         <v>2</v>
       </c>
       <c r="C11" s="57" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D11" s="38" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E11" s="39" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="F11" s="38" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="G11" s="39" t="s">
-        <v>110</v>
-      </c>
-      <c r="H11" s="38"/>
-      <c r="I11" s="38" t="s">
-        <v>139</v>
+        <v>104</v>
+      </c>
+      <c r="H11" s="38" t="s">
+        <v>132</v>
+      </c>
+      <c r="I11" s="36" t="s">
+        <v>168</v>
       </c>
       <c r="J11" s="38" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="K11" s="38">
         <v>1</v>
@@ -1876,7 +1881,7 @@
         <v>5</v>
       </c>
       <c r="M11" s="60" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="N11" s="62"/>
       <c r="O11" s="61">
@@ -1892,26 +1897,28 @@
         <v>3</v>
       </c>
       <c r="C12" s="57" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D12" s="36" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E12" s="37" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="F12" s="36" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="G12" s="37" t="s">
-        <v>111</v>
-      </c>
-      <c r="H12" s="36"/>
+        <v>105</v>
+      </c>
+      <c r="H12" s="36" t="s">
+        <v>133</v>
+      </c>
       <c r="I12" s="36" t="s">
-        <v>140</v>
+        <v>168</v>
       </c>
       <c r="J12" s="36" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="K12" s="36">
         <v>1</v>
@@ -1921,7 +1928,7 @@
         <v>5</v>
       </c>
       <c r="M12" s="59" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="N12" s="61">
         <v>0.1</v>
@@ -1939,26 +1946,28 @@
         <v>4</v>
       </c>
       <c r="C13" s="57" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D13" s="38" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E13" s="39" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="F13" s="38" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="G13" s="39" t="s">
-        <v>112</v>
-      </c>
-      <c r="H13" s="38"/>
-      <c r="I13" s="38" t="s">
-        <v>141</v>
+        <v>106</v>
+      </c>
+      <c r="H13" s="38" t="s">
+        <v>134</v>
+      </c>
+      <c r="I13" s="36" t="s">
+        <v>168</v>
       </c>
       <c r="J13" s="38" t="s">
-        <v>161</v>
+        <v>152</v>
       </c>
       <c r="K13" s="38">
         <v>8</v>
@@ -1968,7 +1977,7 @@
         <v>40</v>
       </c>
       <c r="M13" s="60" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="N13" s="62">
         <v>0.1</v>
@@ -1979,33 +1988,35 @@
       </c>
       <c r="P13" s="38"/>
     </row>
-    <row r="14" spans="1:16" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="50">
         <f>ROW(B14) - ROW($B$9)</f>
         <v>5</v>
       </c>
       <c r="C14" s="56" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D14" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="E14" s="37" t="s">
-        <v>60</v>
+        <v>25</v>
+      </c>
+      <c r="E14" s="36" t="s">
+        <v>185</v>
       </c>
       <c r="F14" s="36" t="s">
-        <v>178</v>
-      </c>
-      <c r="G14" s="37" t="s">
-        <v>91</v>
-      </c>
-      <c r="H14" s="36"/>
+        <v>186</v>
+      </c>
+      <c r="G14" s="36" t="s">
+        <v>187</v>
+      </c>
+      <c r="H14" s="36" t="s">
+        <v>188</v>
+      </c>
       <c r="I14" s="36" t="s">
-        <v>142</v>
+        <v>168</v>
       </c>
       <c r="J14" s="36" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
       <c r="K14" s="36">
         <v>1</v>
@@ -2015,12 +2026,14 @@
         <v>5</v>
       </c>
       <c r="M14" s="60" t="s">
-        <v>190</v>
-      </c>
-      <c r="N14" s="61"/>
+        <v>173</v>
+      </c>
+      <c r="N14" s="61">
+        <v>1.04</v>
+      </c>
       <c r="O14" s="61">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>5.2</v>
       </c>
       <c r="P14" s="36"/>
     </row>
@@ -2031,26 +2044,28 @@
         <v>6</v>
       </c>
       <c r="C15" s="56" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D15" s="38" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E15" s="39" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="F15" s="38" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="G15" s="39" t="s">
-        <v>113</v>
-      </c>
-      <c r="H15" s="38"/>
-      <c r="I15" s="38" t="s">
-        <v>141</v>
+        <v>107</v>
+      </c>
+      <c r="H15" s="38" t="s">
+        <v>134</v>
+      </c>
+      <c r="I15" s="36" t="s">
+        <v>168</v>
       </c>
       <c r="J15" s="38" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="K15" s="38">
         <v>1</v>
@@ -2060,7 +2075,7 @@
         <v>5</v>
       </c>
       <c r="M15" s="60" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="N15" s="62">
         <v>0.1</v>
@@ -2078,26 +2093,28 @@
         <v>7</v>
       </c>
       <c r="C16" s="56" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D16" s="36" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E16" s="37" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="F16" s="36" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="G16" s="37" t="s">
-        <v>114</v>
-      </c>
-      <c r="H16" s="36"/>
+        <v>108</v>
+      </c>
+      <c r="H16" s="36" t="s">
+        <v>134</v>
+      </c>
       <c r="I16" s="36" t="s">
-        <v>141</v>
+        <v>168</v>
       </c>
       <c r="J16" s="36" t="s">
-        <v>164</v>
+        <v>155</v>
       </c>
       <c r="K16" s="36">
         <v>3</v>
@@ -2107,7 +2124,7 @@
         <v>15</v>
       </c>
       <c r="M16" s="59" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="N16" s="61">
         <v>0.1</v>
@@ -2125,26 +2142,28 @@
         <v>8</v>
       </c>
       <c r="C17" s="57" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D17" s="38" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E17" s="39" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="F17" s="38" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="G17" s="39" t="s">
-        <v>115</v>
-      </c>
-      <c r="H17" s="38"/>
-      <c r="I17" s="38" t="s">
-        <v>143</v>
+        <v>109</v>
+      </c>
+      <c r="H17" s="38" t="s">
+        <v>135</v>
+      </c>
+      <c r="I17" s="36" t="s">
+        <v>168</v>
       </c>
       <c r="J17" s="38" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
       <c r="K17" s="38">
         <v>2</v>
@@ -2154,7 +2173,7 @@
         <v>10</v>
       </c>
       <c r="M17" s="59" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="N17" s="62">
         <v>0.11</v>
@@ -2172,26 +2191,28 @@
         <v>9</v>
       </c>
       <c r="C18" s="56" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D18" s="36" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E18" s="37" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="F18" s="36" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="G18" s="37" t="s">
-        <v>116</v>
-      </c>
-      <c r="H18" s="36"/>
+        <v>110</v>
+      </c>
+      <c r="H18" s="36" t="s">
+        <v>136</v>
+      </c>
       <c r="I18" s="36" t="s">
-        <v>144</v>
+        <v>168</v>
       </c>
       <c r="J18" s="36" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="K18" s="36">
         <v>1</v>
@@ -2201,7 +2222,7 @@
         <v>5</v>
       </c>
       <c r="M18" s="59" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="N18" s="61">
         <v>0.23</v>
@@ -2219,26 +2240,28 @@
         <v>10</v>
       </c>
       <c r="C19" s="57" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D19" s="38" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E19" s="39" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="F19" s="38" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="G19" s="39" t="s">
-        <v>117</v>
-      </c>
-      <c r="H19" s="38"/>
-      <c r="I19" s="38" t="s">
-        <v>145</v>
+        <v>111</v>
+      </c>
+      <c r="H19" s="38" t="s">
+        <v>137</v>
+      </c>
+      <c r="I19" s="36" t="s">
+        <v>168</v>
       </c>
       <c r="J19" s="38" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="K19" s="38">
         <v>2</v>
@@ -2248,7 +2271,7 @@
         <v>10</v>
       </c>
       <c r="M19" s="60" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="N19" s="62"/>
       <c r="O19" s="61">
@@ -2264,26 +2287,28 @@
         <v>11</v>
       </c>
       <c r="C20" s="56" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D20" s="36" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E20" s="37" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="F20" s="36" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="G20" s="37" t="s">
-        <v>118</v>
-      </c>
-      <c r="H20" s="36"/>
+        <v>112</v>
+      </c>
+      <c r="H20" s="36" t="s">
+        <v>138</v>
+      </c>
       <c r="I20" s="36" t="s">
-        <v>146</v>
+        <v>168</v>
       </c>
       <c r="J20" s="36" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="K20" s="36">
         <v>1</v>
@@ -2293,7 +2318,7 @@
         <v>5</v>
       </c>
       <c r="M20" s="59" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="N20" s="61">
         <v>0.48</v>
@@ -2311,26 +2336,28 @@
         <v>12</v>
       </c>
       <c r="C21" s="57" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D21" s="38" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E21" s="39" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="F21" s="38" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="G21" s="39" t="s">
-        <v>119</v>
-      </c>
-      <c r="H21" s="38"/>
-      <c r="I21" s="38" t="s">
-        <v>147</v>
+        <v>113</v>
+      </c>
+      <c r="H21" s="38" t="s">
+        <v>139</v>
+      </c>
+      <c r="I21" s="36" t="s">
+        <v>168</v>
       </c>
       <c r="J21" s="38" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="K21" s="38">
         <v>1</v>
@@ -2340,7 +2367,7 @@
         <v>5</v>
       </c>
       <c r="M21" s="60" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="N21" s="62"/>
       <c r="O21" s="61">
@@ -2356,26 +2383,28 @@
         <v>13</v>
       </c>
       <c r="C22" s="56" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D22" s="36" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E22" s="37" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="F22" s="36" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="G22" s="37" t="s">
-        <v>120</v>
-      </c>
-      <c r="H22" s="36"/>
+        <v>114</v>
+      </c>
+      <c r="H22" s="36" t="s">
+        <v>140</v>
+      </c>
       <c r="I22" s="36" t="s">
-        <v>148</v>
+        <v>168</v>
       </c>
       <c r="J22" s="36" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="K22" s="36">
         <v>1</v>
@@ -2385,7 +2414,7 @@
         <v>5</v>
       </c>
       <c r="M22" s="60" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="N22" s="61"/>
       <c r="O22" s="61">
@@ -2394,33 +2423,35 @@
       </c>
       <c r="P22" s="36"/>
     </row>
-    <row r="23" spans="1:16" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:16" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="50">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="C23" s="57" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D23" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="E23" s="39" t="s">
-        <v>69</v>
+        <v>34</v>
+      </c>
+      <c r="E23" s="38" t="s">
+        <v>182</v>
       </c>
       <c r="F23" s="38" t="s">
-        <v>178</v>
-      </c>
-      <c r="G23" s="39" t="s">
-        <v>121</v>
-      </c>
-      <c r="H23" s="38"/>
-      <c r="I23" s="38" t="s">
-        <v>149</v>
+        <v>169</v>
+      </c>
+      <c r="G23" s="38" t="s">
+        <v>183</v>
+      </c>
+      <c r="H23" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="I23" s="36" t="s">
+        <v>168</v>
       </c>
       <c r="J23" s="38" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="K23" s="38">
         <v>1</v>
@@ -2429,15 +2460,13 @@
         <f t="shared" ref="L23" si="8">K23*5</f>
         <v>5</v>
       </c>
-      <c r="M23" s="59" t="s">
-        <v>182</v>
-      </c>
-      <c r="N23" s="62">
-        <v>1.69</v>
-      </c>
+      <c r="M23" s="60" t="s">
+        <v>181</v>
+      </c>
+      <c r="N23" s="62"/>
       <c r="O23" s="61">
         <f t="shared" si="2"/>
-        <v>8.4499999999999993</v>
+        <v>0</v>
       </c>
       <c r="P23" s="38"/>
     </row>
@@ -2448,28 +2477,28 @@
         <v>15</v>
       </c>
       <c r="C24" s="56" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
       <c r="D24" s="36" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E24" s="37" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="F24" s="55" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="G24" s="37" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="H24" s="36" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="I24" s="36" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="J24" s="55" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="K24" s="36">
         <v>1</v>
@@ -2479,7 +2508,7 @@
         <v>5</v>
       </c>
       <c r="M24" s="55" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="N24" s="61"/>
       <c r="O24" s="61">
@@ -2495,28 +2524,28 @@
         <v>16</v>
       </c>
       <c r="C25" s="57" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D25" s="38" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E25" s="39" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="F25" s="38" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="G25" s="39" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="H25" s="36" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="I25" s="36" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="J25" s="55" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="K25" s="38">
         <v>1</v>
@@ -2526,7 +2555,7 @@
         <v>5</v>
       </c>
       <c r="M25" s="55" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="N25" s="62"/>
       <c r="O25" s="61">
@@ -2542,28 +2571,28 @@
         <v>17</v>
       </c>
       <c r="C26" s="56" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D26" s="36" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E26" s="37" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="F26" s="36" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="G26" s="37" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="H26" s="36" t="s">
-        <v>177</v>
+        <v>141</v>
       </c>
       <c r="I26" s="36" t="s">
-        <v>150</v>
+        <v>168</v>
       </c>
       <c r="J26" s="36" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="K26" s="36">
         <v>1</v>
@@ -2573,7 +2602,7 @@
         <v>5</v>
       </c>
       <c r="M26" s="60" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="N26" s="61"/>
       <c r="O26" s="61">
@@ -2589,26 +2618,28 @@
         <v>18</v>
       </c>
       <c r="C27" s="57" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D27" s="38" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E27" s="39" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F27" s="38" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="G27" s="39" t="s">
-        <v>123</v>
-      </c>
-      <c r="H27" s="38"/>
-      <c r="I27" s="38" t="s">
-        <v>139</v>
+        <v>116</v>
+      </c>
+      <c r="H27" s="38" t="s">
+        <v>132</v>
+      </c>
+      <c r="I27" s="36" t="s">
+        <v>168</v>
       </c>
       <c r="J27" s="38" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
       <c r="K27" s="38">
         <v>1</v>
@@ -2618,7 +2649,7 @@
         <v>5</v>
       </c>
       <c r="M27" s="60" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="N27" s="62"/>
       <c r="O27" s="61">
@@ -2634,26 +2665,28 @@
         <v>19</v>
       </c>
       <c r="C28" s="56" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D28" s="36" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E28" s="37" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F28" s="36" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="G28" s="37" t="s">
-        <v>124</v>
-      </c>
-      <c r="H28" s="36"/>
+        <v>117</v>
+      </c>
+      <c r="H28" s="36" t="s">
+        <v>142</v>
+      </c>
       <c r="I28" s="36" t="s">
-        <v>151</v>
+        <v>168</v>
       </c>
       <c r="J28" s="36" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="K28" s="36">
         <v>1</v>
@@ -2663,7 +2696,7 @@
         <v>5</v>
       </c>
       <c r="M28" s="60" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="N28" s="61"/>
       <c r="O28" s="61">
@@ -2679,26 +2712,28 @@
         <v>20</v>
       </c>
       <c r="C29" s="57" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D29" s="38" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E29" s="39" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="F29" s="38" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="G29" s="39" t="s">
-        <v>125</v>
-      </c>
-      <c r="H29" s="38"/>
-      <c r="I29" s="38" t="s">
-        <v>151</v>
+        <v>118</v>
+      </c>
+      <c r="H29" s="38" t="s">
+        <v>142</v>
+      </c>
+      <c r="I29" s="36" t="s">
+        <v>168</v>
       </c>
       <c r="J29" s="38" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="K29" s="38">
         <v>1</v>
@@ -2708,7 +2743,7 @@
         <v>5</v>
       </c>
       <c r="M29" s="60" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="N29" s="62"/>
       <c r="O29" s="61">
@@ -2724,26 +2759,28 @@
         <v>21</v>
       </c>
       <c r="C30" s="56" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D30" s="36" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E30" s="37" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="F30" s="36" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="G30" s="37" t="s">
-        <v>126</v>
-      </c>
-      <c r="H30" s="36"/>
+        <v>119</v>
+      </c>
+      <c r="H30" s="36" t="s">
+        <v>143</v>
+      </c>
       <c r="I30" s="36" t="s">
-        <v>152</v>
+        <v>168</v>
       </c>
       <c r="J30" s="36" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="K30" s="36">
         <v>4</v>
@@ -2753,7 +2790,7 @@
         <v>20</v>
       </c>
       <c r="M30" s="60" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="N30" s="61"/>
       <c r="O30" s="61">
@@ -2769,28 +2806,28 @@
         <v>22</v>
       </c>
       <c r="C31" s="57" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D31" s="38" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E31" s="39" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="F31" s="38" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="G31" s="39" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="H31" s="38" t="s">
-        <v>177</v>
-      </c>
-      <c r="I31" s="38" t="s">
-        <v>141</v>
+        <v>134</v>
+      </c>
+      <c r="I31" s="36" t="s">
+        <v>168</v>
       </c>
       <c r="J31" s="38" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="K31" s="38">
         <v>3</v>
@@ -2800,7 +2837,7 @@
         <v>15</v>
       </c>
       <c r="M31" s="59" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="N31" s="62">
         <v>0.1</v>
@@ -2818,26 +2855,28 @@
         <v>23</v>
       </c>
       <c r="C32" s="56" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D32" s="36" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E32" s="37" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="F32" s="36" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="G32" s="37" t="s">
-        <v>128</v>
-      </c>
-      <c r="H32" s="36"/>
+        <v>121</v>
+      </c>
+      <c r="H32" s="36" t="s">
+        <v>134</v>
+      </c>
       <c r="I32" s="36" t="s">
-        <v>141</v>
+        <v>168</v>
       </c>
       <c r="J32" s="36" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="K32" s="36">
         <v>2</v>
@@ -2847,7 +2886,7 @@
         <v>10</v>
       </c>
       <c r="M32" s="59" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="N32" s="62">
         <v>0.1</v>
@@ -2865,26 +2904,28 @@
         <v>24</v>
       </c>
       <c r="C33" s="57" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D33" s="38" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E33" s="39" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="F33" s="38" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="G33" s="39" t="s">
-        <v>129</v>
-      </c>
-      <c r="H33" s="38"/>
-      <c r="I33" s="38" t="s">
-        <v>141</v>
+        <v>122</v>
+      </c>
+      <c r="H33" s="38" t="s">
+        <v>134</v>
+      </c>
+      <c r="I33" s="36" t="s">
+        <v>168</v>
       </c>
       <c r="J33" s="38" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="K33" s="38">
         <v>2</v>
@@ -2894,7 +2935,7 @@
         <v>10</v>
       </c>
       <c r="M33" s="59" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="N33" s="62">
         <v>0.1</v>
@@ -2912,26 +2953,28 @@
         <v>25</v>
       </c>
       <c r="C34" s="56" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D34" s="36" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E34" s="37" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="F34" s="36" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="G34" s="37" t="s">
-        <v>130</v>
-      </c>
-      <c r="H34" s="36"/>
+        <v>123</v>
+      </c>
+      <c r="H34" s="36" t="s">
+        <v>134</v>
+      </c>
       <c r="I34" s="36" t="s">
-        <v>141</v>
+        <v>168</v>
       </c>
       <c r="J34" s="36" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="K34" s="36">
         <v>4</v>
@@ -2941,7 +2984,7 @@
         <v>20</v>
       </c>
       <c r="M34" s="59" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="N34" s="62">
         <v>0.1</v>
@@ -2959,26 +3002,28 @@
         <v>26</v>
       </c>
       <c r="C35" s="56" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D35" s="38" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E35" s="39" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F35" s="38" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="G35" s="39" t="s">
-        <v>131</v>
-      </c>
-      <c r="H35" s="38"/>
-      <c r="I35" s="38" t="s">
-        <v>141</v>
+        <v>124</v>
+      </c>
+      <c r="H35" s="38" t="s">
+        <v>134</v>
+      </c>
+      <c r="I35" s="36" t="s">
+        <v>168</v>
       </c>
       <c r="J35" s="38" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="K35" s="38">
         <v>4</v>
@@ -2988,7 +3033,7 @@
         <v>20</v>
       </c>
       <c r="M35" s="59" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="N35" s="62">
         <v>0.1</v>
@@ -3006,43 +3051,45 @@
         <v>27</v>
       </c>
       <c r="C36" s="56" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D36" s="36" t="s">
-        <v>49</v>
+        <v>189</v>
       </c>
       <c r="E36" s="37" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="F36" s="36" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="G36" s="37" t="s">
-        <v>132</v>
-      </c>
-      <c r="H36" s="36"/>
+        <v>125</v>
+      </c>
+      <c r="H36" s="36" t="s">
+        <v>134</v>
+      </c>
       <c r="I36" s="36" t="s">
-        <v>141</v>
+        <v>168</v>
       </c>
       <c r="J36" s="36" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="K36" s="36">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L36" s="36">
         <f>K36*5</f>
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="M36" s="59" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="N36" s="62">
         <v>0.1</v>
       </c>
       <c r="O36" s="63">
         <f t="shared" si="13"/>
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="P36" s="36"/>
     </row>
@@ -3053,28 +3100,28 @@
         <v>28</v>
       </c>
       <c r="C37" s="57" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D37" s="38" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="E37" s="39" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="F37" s="38" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="G37" s="39" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="H37" s="38" t="s">
-        <v>177</v>
-      </c>
-      <c r="I37" s="38" t="s">
-        <v>153</v>
+        <v>144</v>
+      </c>
+      <c r="I37" s="36" t="s">
+        <v>168</v>
       </c>
       <c r="J37" s="38" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="K37" s="38">
         <v>1</v>
@@ -3084,7 +3131,7 @@
         <v>5</v>
       </c>
       <c r="M37" s="60" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="N37" s="62"/>
       <c r="O37" s="63">
@@ -3100,26 +3147,28 @@
         <v>29</v>
       </c>
       <c r="C38" s="56" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D38" s="36" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E38" s="37" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="F38" s="36" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="G38" s="37" t="s">
-        <v>133</v>
-      </c>
-      <c r="H38" s="36"/>
+        <v>126</v>
+      </c>
+      <c r="H38" s="36" t="s">
+        <v>145</v>
+      </c>
       <c r="I38" s="36" t="s">
-        <v>154</v>
+        <v>168</v>
       </c>
       <c r="J38" s="36" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="K38" s="36">
         <v>1</v>
@@ -3129,7 +3178,7 @@
         <v>5</v>
       </c>
       <c r="M38" s="59" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="N38" s="61">
         <v>0.95</v>
@@ -3147,23 +3196,25 @@
         <v>30</v>
       </c>
       <c r="C39" s="57" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D39" s="38" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="E39" s="39" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="F39" s="38" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="G39" s="39" t="s">
-        <v>134</v>
-      </c>
-      <c r="H39" s="38"/>
-      <c r="I39" s="38" t="s">
-        <v>155</v>
+        <v>127</v>
+      </c>
+      <c r="H39" s="38" t="s">
+        <v>146</v>
+      </c>
+      <c r="I39" s="36" t="s">
+        <v>168</v>
       </c>
       <c r="J39" s="38"/>
       <c r="K39" s="38">
@@ -3174,7 +3225,7 @@
         <v>5</v>
       </c>
       <c r="M39" s="59" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="N39" s="62"/>
       <c r="O39" s="63">
@@ -3190,26 +3241,28 @@
         <v>31</v>
       </c>
       <c r="C40" s="56" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D40" s="36" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E40" s="37" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="F40" s="36" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="G40" s="37" t="s">
-        <v>135</v>
-      </c>
-      <c r="H40" s="36"/>
+        <v>128</v>
+      </c>
+      <c r="H40" s="36" t="s">
+        <v>147</v>
+      </c>
       <c r="I40" s="36" t="s">
-        <v>156</v>
+        <v>168</v>
       </c>
       <c r="J40" s="36" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="K40" s="36">
         <v>1</v>
@@ -3219,7 +3272,7 @@
         <v>5</v>
       </c>
       <c r="M40" s="60" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="N40" s="61"/>
       <c r="O40" s="63">
@@ -3235,26 +3288,28 @@
         <v>32</v>
       </c>
       <c r="C41" s="57" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D41" s="38" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E41" s="39" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="F41" s="38" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="G41" s="39" t="s">
-        <v>136</v>
-      </c>
-      <c r="H41" s="38"/>
-      <c r="I41" s="38" t="s">
-        <v>157</v>
+        <v>129</v>
+      </c>
+      <c r="H41" s="38" t="s">
+        <v>148</v>
+      </c>
+      <c r="I41" s="36" t="s">
+        <v>168</v>
       </c>
       <c r="J41" s="38" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="K41" s="38">
         <v>1</v>
@@ -3264,7 +3319,7 @@
         <v>5</v>
       </c>
       <c r="M41" s="59" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="N41" s="62">
         <v>1.08</v>
@@ -3282,22 +3337,24 @@
         <v>33</v>
       </c>
       <c r="C42" s="57" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
       <c r="D42" s="38" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="E42" s="38" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="F42" s="38" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="G42" s="38" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="H42" s="38"/>
-      <c r="I42" s="38"/>
+      <c r="I42" s="36" t="s">
+        <v>168</v>
+      </c>
       <c r="J42" s="38"/>
       <c r="K42" s="38">
         <v>1</v>
@@ -3307,7 +3364,7 @@
         <v>5</v>
       </c>
       <c r="M42" s="59" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
       <c r="N42" s="62">
         <v>0.8</v>
@@ -3325,14 +3382,16 @@
         <v>34</v>
       </c>
       <c r="C43" s="57" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
       <c r="D43" s="64"/>
       <c r="E43" s="64"/>
       <c r="F43" s="64"/>
       <c r="G43" s="64"/>
       <c r="H43" s="64"/>
-      <c r="I43" s="64"/>
+      <c r="I43" s="36" t="s">
+        <v>168</v>
+      </c>
       <c r="J43" s="64"/>
       <c r="K43" s="64"/>
       <c r="L43" s="64"/>
@@ -3349,18 +3408,18 @@
       <c r="E44" s="33"/>
       <c r="F44" s="34"/>
       <c r="G44" s="35"/>
-      <c r="H44" s="35"/>
-      <c r="I44" s="34"/>
+      <c r="H44" s="34"/>
+      <c r="I44" s="35"/>
       <c r="J44" s="35"/>
       <c r="K44" s="35"/>
       <c r="L44" s="75" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="M44" s="76"/>
       <c r="N44" s="76"/>
       <c r="O44" s="69">
         <f>SUM(O10:O43)</f>
-        <v>47.25</v>
+        <v>44.999999999999993</v>
       </c>
       <c r="P44" s="41"/>
     </row>
@@ -3377,13 +3436,13 @@
       <c r="J45" s="9"/>
       <c r="K45" s="9"/>
       <c r="L45" s="75" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
       <c r="M45" s="76"/>
       <c r="N45" s="76"/>
       <c r="O45" s="70">
         <f>O44/5</f>
-        <v>9.4499999999999993</v>
+        <v>8.9999999999999982</v>
       </c>
       <c r="P45" s="42"/>
     </row>
@@ -3396,24 +3455,24 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="M10" r:id="rId1"/>
-    <hyperlink ref="M23" r:id="rId2"/>
-    <hyperlink ref="M12" r:id="rId3"/>
-    <hyperlink ref="M13" r:id="rId4"/>
-    <hyperlink ref="M15" r:id="rId5"/>
-    <hyperlink ref="M16" r:id="rId6"/>
-    <hyperlink ref="M17" r:id="rId7"/>
-    <hyperlink ref="M18" r:id="rId8"/>
-    <hyperlink ref="M20" r:id="rId9"/>
-    <hyperlink ref="M31" r:id="rId10"/>
-    <hyperlink ref="M32" r:id="rId11"/>
-    <hyperlink ref="M33" r:id="rId12"/>
-    <hyperlink ref="M34" r:id="rId13"/>
-    <hyperlink ref="M35" r:id="rId14"/>
-    <hyperlink ref="M36" r:id="rId15"/>
-    <hyperlink ref="M38" r:id="rId16"/>
-    <hyperlink ref="M39" r:id="rId17"/>
-    <hyperlink ref="M41" r:id="rId18"/>
-    <hyperlink ref="M42" r:id="rId19"/>
+    <hyperlink ref="M12" r:id="rId2"/>
+    <hyperlink ref="M13" r:id="rId3"/>
+    <hyperlink ref="M15" r:id="rId4"/>
+    <hyperlink ref="M16" r:id="rId5"/>
+    <hyperlink ref="M17" r:id="rId6"/>
+    <hyperlink ref="M18" r:id="rId7"/>
+    <hyperlink ref="M20" r:id="rId8"/>
+    <hyperlink ref="M31" r:id="rId9"/>
+    <hyperlink ref="M32" r:id="rId10"/>
+    <hyperlink ref="M33" r:id="rId11"/>
+    <hyperlink ref="M34" r:id="rId12"/>
+    <hyperlink ref="M35" r:id="rId13"/>
+    <hyperlink ref="M36" r:id="rId14"/>
+    <hyperlink ref="M38" r:id="rId15"/>
+    <hyperlink ref="M39" r:id="rId16"/>
+    <hyperlink ref="M41" r:id="rId17"/>
+    <hyperlink ref="M42" r:id="rId18"/>
+    <hyperlink ref="M14" r:id="rId19"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId20"/>

</xml_diff>

<commit_message>
#16 BOM update according to design CHanges.
</commit_message>
<xml_diff>
--- a/Design Files/LTE-Module-v2.0/BOM/Client_BOM_v2.0.xlsx
+++ b/Design Files/LTE-Module-v2.0/BOM/Client_BOM_v2.0.xlsx
@@ -93,9 +93,6 @@
     <t>C2</t>
   </si>
   <si>
-    <t>C3, C4, C5, C11, C13, C15, C16, C17</t>
-  </si>
-  <si>
     <t>C6</t>
   </si>
   <si>
@@ -595,6 +592,9 @@
   </si>
   <si>
     <t>LTE_MODULE_v2.0</t>
+  </si>
+  <si>
+    <t>C5, C11, C13, C15, C16, C17</t>
   </si>
 </sst>
 </file>
@@ -1013,7 +1013,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1181,21 +1181,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="17" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="17" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="14" fillId="3" borderId="14" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1596,13 +1581,13 @@
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
-      <c r="J1" s="72"/>
-      <c r="K1" s="72"/>
-      <c r="L1" s="72"/>
-      <c r="M1" s="72"/>
-      <c r="N1" s="72"/>
-      <c r="O1" s="72"/>
-      <c r="P1" s="72"/>
+      <c r="J1" s="67"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="67"/>
     </row>
     <row r="2" spans="1:16" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1613,7 +1598,7 @@
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="51" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="3"/>
@@ -1635,7 +1620,7 @@
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="52" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="4"/>
@@ -1646,7 +1631,7 @@
       <c r="M3" s="4"/>
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
-      <c r="P3" s="73"/>
+      <c r="P3" s="68"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1657,7 +1642,7 @@
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="53" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G4" s="13"/>
       <c r="H4" s="6"/>
@@ -1668,7 +1653,7 @@
       <c r="M4" s="58"/>
       <c r="N4" s="58"/>
       <c r="O4" s="58"/>
-      <c r="P4" s="74"/>
+      <c r="P4" s="69"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1690,7 +1675,7 @@
       <c r="M5" s="58"/>
       <c r="N5" s="58"/>
       <c r="O5" s="58"/>
-      <c r="P5" s="74"/>
+      <c r="P5" s="69"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -1708,7 +1693,7 @@
       <c r="M6" s="58"/>
       <c r="N6" s="58"/>
       <c r="O6" s="58"/>
-      <c r="P6" s="74"/>
+      <c r="P6" s="69"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -1726,7 +1711,7 @@
       <c r="M7" s="7"/>
       <c r="N7" s="7"/>
       <c r="O7" s="7"/>
-      <c r="P7" s="74"/>
+      <c r="P7" s="69"/>
     </row>
     <row r="8" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1744,7 +1729,7 @@
       <c r="M8" s="7"/>
       <c r="N8" s="7"/>
       <c r="O8" s="7"/>
-      <c r="P8" s="74"/>
+      <c r="P8" s="69"/>
     </row>
     <row r="9" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -1758,40 +1743,40 @@
         <v>20</v>
       </c>
       <c r="E9" s="30" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F9" s="29" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G9" s="30" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H9" s="29" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I9" s="29" t="s">
+        <v>164</v>
+      </c>
+      <c r="J9" s="29" t="s">
+        <v>166</v>
+      </c>
+      <c r="K9" s="29" t="s">
+        <v>163</v>
+      </c>
+      <c r="L9" s="29" t="s">
         <v>165</v>
       </c>
-      <c r="J9" s="29" t="s">
-        <v>167</v>
-      </c>
-      <c r="K9" s="29" t="s">
-        <v>164</v>
-      </c>
-      <c r="L9" s="29" t="s">
-        <v>166</v>
-      </c>
       <c r="M9" s="29" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="N9" s="29" t="s">
+        <v>173</v>
+      </c>
+      <c r="O9" s="29" t="s">
         <v>174</v>
       </c>
-      <c r="O9" s="29" t="s">
-        <v>175</v>
-      </c>
       <c r="P9" s="29" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1807,22 +1792,22 @@
         <v>21</v>
       </c>
       <c r="E10" s="37" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F10" s="36" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G10" s="37" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H10" s="36" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="I10" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J10" s="36" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="K10" s="36">
         <v>1</v>
@@ -1832,7 +1817,7 @@
         <v>5</v>
       </c>
       <c r="M10" s="59" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="N10" s="61">
         <v>0.9</v>
@@ -1856,22 +1841,22 @@
         <v>22</v>
       </c>
       <c r="E11" s="39" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F11" s="38" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G11" s="39" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H11" s="38" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="I11" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J11" s="38" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="K11" s="38">
         <v>1</v>
@@ -1881,7 +1866,7 @@
         <v>5</v>
       </c>
       <c r="M11" s="60" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="N11" s="62"/>
       <c r="O11" s="61">
@@ -1903,22 +1888,22 @@
         <v>23</v>
       </c>
       <c r="E12" s="37" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F12" s="36" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G12" s="37" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H12" s="36" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I12" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J12" s="36" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K12" s="36">
         <v>1</v>
@@ -1928,7 +1913,7 @@
         <v>5</v>
       </c>
       <c r="M12" s="59" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="N12" s="61">
         <v>0.1</v>
@@ -1949,42 +1934,42 @@
         <v>8</v>
       </c>
       <c r="D13" s="38" t="s">
-        <v>24</v>
+        <v>191</v>
       </c>
       <c r="E13" s="39" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F13" s="38" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G13" s="39" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H13" s="38" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I13" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J13" s="38" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K13" s="38">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L13" s="38">
         <f t="shared" ref="L13" si="3">K13*5</f>
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="M13" s="60" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="N13" s="62">
         <v>0.1</v>
       </c>
       <c r="O13" s="61">
         <f t="shared" si="2"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P13" s="38"/>
     </row>
@@ -1998,25 +1983,25 @@
         <v>8</v>
       </c>
       <c r="D14" s="36" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E14" s="36" t="s">
+        <v>184</v>
+      </c>
+      <c r="F14" s="36" t="s">
         <v>185</v>
       </c>
-      <c r="F14" s="36" t="s">
+      <c r="G14" s="36" t="s">
         <v>186</v>
       </c>
-      <c r="G14" s="36" t="s">
+      <c r="H14" s="36" t="s">
         <v>187</v>
       </c>
-      <c r="H14" s="36" t="s">
-        <v>188</v>
-      </c>
       <c r="I14" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J14" s="36" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="K14" s="36">
         <v>1</v>
@@ -2026,7 +2011,7 @@
         <v>5</v>
       </c>
       <c r="M14" s="60" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="N14" s="61">
         <v>1.04</v>
@@ -2047,25 +2032,25 @@
         <v>8</v>
       </c>
       <c r="D15" s="38" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E15" s="39" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F15" s="38" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G15" s="39" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H15" s="38" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I15" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J15" s="38" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K15" s="38">
         <v>1</v>
@@ -2075,7 +2060,7 @@
         <v>5</v>
       </c>
       <c r="M15" s="60" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="N15" s="62">
         <v>0.1</v>
@@ -2096,25 +2081,25 @@
         <v>8</v>
       </c>
       <c r="D16" s="36" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E16" s="37" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F16" s="36" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G16" s="37" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H16" s="36" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I16" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J16" s="36" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K16" s="36">
         <v>3</v>
@@ -2124,7 +2109,7 @@
         <v>15</v>
       </c>
       <c r="M16" s="59" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="N16" s="61">
         <v>0.1</v>
@@ -2145,25 +2130,25 @@
         <v>8</v>
       </c>
       <c r="D17" s="38" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E17" s="39" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F17" s="38" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G17" s="39" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H17" s="38" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I17" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J17" s="38" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="K17" s="38">
         <v>2</v>
@@ -2173,7 +2158,7 @@
         <v>10</v>
       </c>
       <c r="M17" s="59" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="N17" s="62">
         <v>0.11</v>
@@ -2194,25 +2179,25 @@
         <v>9</v>
       </c>
       <c r="D18" s="36" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E18" s="37" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F18" s="36" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G18" s="37" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H18" s="36" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I18" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J18" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="K18" s="36">
         <v>1</v>
@@ -2222,7 +2207,7 @@
         <v>5</v>
       </c>
       <c r="M18" s="59" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="N18" s="61">
         <v>0.23</v>
@@ -2243,25 +2228,25 @@
         <v>9</v>
       </c>
       <c r="D19" s="38" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E19" s="39" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F19" s="38" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G19" s="39" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H19" s="38" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I19" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J19" s="38" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="K19" s="38">
         <v>2</v>
@@ -2271,7 +2256,7 @@
         <v>10</v>
       </c>
       <c r="M19" s="60" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="N19" s="62"/>
       <c r="O19" s="61">
@@ -2290,25 +2275,25 @@
         <v>9</v>
       </c>
       <c r="D20" s="36" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E20" s="37" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F20" s="36" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G20" s="37" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H20" s="36" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I20" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J20" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="K20" s="36">
         <v>1</v>
@@ -2318,7 +2303,7 @@
         <v>5</v>
       </c>
       <c r="M20" s="59" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="N20" s="61">
         <v>0.48</v>
@@ -2339,25 +2324,25 @@
         <v>9</v>
       </c>
       <c r="D21" s="38" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E21" s="39" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F21" s="38" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G21" s="39" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H21" s="38" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I21" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J21" s="38" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="K21" s="38">
         <v>1</v>
@@ -2367,7 +2352,7 @@
         <v>5</v>
       </c>
       <c r="M21" s="60" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="N21" s="62"/>
       <c r="O21" s="61">
@@ -2386,25 +2371,25 @@
         <v>10</v>
       </c>
       <c r="D22" s="36" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E22" s="37" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F22" s="36" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G22" s="37" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H22" s="36" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="I22" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J22" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="K22" s="36">
         <v>1</v>
@@ -2414,7 +2399,7 @@
         <v>5</v>
       </c>
       <c r="M22" s="60" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="N22" s="61"/>
       <c r="O22" s="61">
@@ -2433,25 +2418,25 @@
         <v>11</v>
       </c>
       <c r="D23" s="38" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E23" s="38" t="s">
+        <v>181</v>
+      </c>
+      <c r="F23" s="38" t="s">
+        <v>168</v>
+      </c>
+      <c r="G23" s="38" t="s">
         <v>182</v>
       </c>
-      <c r="F23" s="38" t="s">
-        <v>169</v>
-      </c>
-      <c r="G23" s="38" t="s">
+      <c r="H23" s="38" t="s">
         <v>183</v>
       </c>
-      <c r="H23" s="38" t="s">
-        <v>184</v>
-      </c>
       <c r="I23" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J23" s="38" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="K23" s="38">
         <v>1</v>
@@ -2461,7 +2446,7 @@
         <v>5</v>
       </c>
       <c r="M23" s="60" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="N23" s="62"/>
       <c r="O23" s="61">
@@ -2477,28 +2462,28 @@
         <v>15</v>
       </c>
       <c r="C24" s="56" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D24" s="36" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E24" s="37" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F24" s="55" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G24" s="37" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H24" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="I24" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J24" s="55" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="K24" s="36">
         <v>1</v>
@@ -2508,7 +2493,7 @@
         <v>5</v>
       </c>
       <c r="M24" s="55" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="N24" s="61"/>
       <c r="O24" s="61">
@@ -2527,25 +2512,25 @@
         <v>12</v>
       </c>
       <c r="D25" s="38" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E25" s="39" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F25" s="38" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G25" s="39" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H25" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="I25" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J25" s="55" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="K25" s="38">
         <v>1</v>
@@ -2555,7 +2540,7 @@
         <v>5</v>
       </c>
       <c r="M25" s="55" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="N25" s="62"/>
       <c r="O25" s="61">
@@ -2574,25 +2559,25 @@
         <v>13</v>
       </c>
       <c r="D26" s="36" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E26" s="37" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F26" s="36" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G26" s="37" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H26" s="36" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="I26" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J26" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="K26" s="36">
         <v>1</v>
@@ -2602,7 +2587,7 @@
         <v>5</v>
       </c>
       <c r="M26" s="60" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="N26" s="61"/>
       <c r="O26" s="61">
@@ -2621,25 +2606,25 @@
         <v>14</v>
       </c>
       <c r="D27" s="38" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E27" s="39" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F27" s="38" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G27" s="39" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H27" s="38" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="I27" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J27" s="38" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="K27" s="38">
         <v>1</v>
@@ -2649,7 +2634,7 @@
         <v>5</v>
       </c>
       <c r="M27" s="60" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="N27" s="62"/>
       <c r="O27" s="61">
@@ -2668,25 +2653,25 @@
         <v>15</v>
       </c>
       <c r="D28" s="36" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E28" s="37" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F28" s="36" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G28" s="37" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H28" s="36" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="I28" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J28" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="K28" s="36">
         <v>1</v>
@@ -2696,7 +2681,7 @@
         <v>5</v>
       </c>
       <c r="M28" s="60" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="N28" s="61"/>
       <c r="O28" s="61">
@@ -2715,25 +2700,25 @@
         <v>15</v>
       </c>
       <c r="D29" s="38" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E29" s="39" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F29" s="38" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G29" s="39" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H29" s="38" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="I29" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J29" s="38" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="K29" s="38">
         <v>1</v>
@@ -2743,7 +2728,7 @@
         <v>5</v>
       </c>
       <c r="M29" s="60" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="N29" s="62"/>
       <c r="O29" s="61">
@@ -2762,25 +2747,25 @@
         <v>16</v>
       </c>
       <c r="D30" s="36" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E30" s="37" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F30" s="36" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G30" s="37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H30" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="I30" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J30" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="K30" s="36">
         <v>4</v>
@@ -2790,7 +2775,7 @@
         <v>20</v>
       </c>
       <c r="M30" s="60" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="N30" s="61"/>
       <c r="O30" s="61">
@@ -2809,25 +2794,25 @@
         <v>17</v>
       </c>
       <c r="D31" s="38" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E31" s="39" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F31" s="38" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G31" s="39" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H31" s="38" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I31" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J31" s="38" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K31" s="38">
         <v>3</v>
@@ -2837,7 +2822,7 @@
         <v>15</v>
       </c>
       <c r="M31" s="59" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="N31" s="62">
         <v>0.1</v>
@@ -2858,25 +2843,25 @@
         <v>17</v>
       </c>
       <c r="D32" s="36" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E32" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F32" s="36" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G32" s="37" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H32" s="36" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I32" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J32" s="36" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K32" s="36">
         <v>2</v>
@@ -2886,7 +2871,7 @@
         <v>10</v>
       </c>
       <c r="M32" s="59" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="N32" s="62">
         <v>0.1</v>
@@ -2907,25 +2892,25 @@
         <v>17</v>
       </c>
       <c r="D33" s="38" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E33" s="39" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F33" s="38" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G33" s="39" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H33" s="38" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I33" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J33" s="38" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="K33" s="38">
         <v>2</v>
@@ -2935,7 +2920,7 @@
         <v>10</v>
       </c>
       <c r="M33" s="59" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="N33" s="62">
         <v>0.1</v>
@@ -2956,25 +2941,25 @@
         <v>17</v>
       </c>
       <c r="D34" s="36" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E34" s="37" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F34" s="36" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G34" s="37" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H34" s="36" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I34" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J34" s="36" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="K34" s="36">
         <v>4</v>
@@ -2984,7 +2969,7 @@
         <v>20</v>
       </c>
       <c r="M34" s="59" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="N34" s="62">
         <v>0.1</v>
@@ -3005,25 +2990,25 @@
         <v>17</v>
       </c>
       <c r="D35" s="38" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E35" s="39" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F35" s="38" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G35" s="39" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H35" s="38" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I35" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J35" s="38" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="K35" s="38">
         <v>4</v>
@@ -3033,7 +3018,7 @@
         <v>20</v>
       </c>
       <c r="M35" s="59" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="N35" s="62">
         <v>0.1</v>
@@ -3054,25 +3039,25 @@
         <v>17</v>
       </c>
       <c r="D36" s="36" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E36" s="37" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F36" s="36" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G36" s="37" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H36" s="36" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I36" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J36" s="36" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="K36" s="36">
         <v>5</v>
@@ -3082,7 +3067,7 @@
         <v>25</v>
       </c>
       <c r="M36" s="59" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="N36" s="62">
         <v>0.1</v>
@@ -3103,25 +3088,25 @@
         <v>18</v>
       </c>
       <c r="D37" s="38" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E37" s="39" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F37" s="38" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G37" s="39" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="H37" s="38" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I37" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J37" s="38" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="K37" s="38">
         <v>1</v>
@@ -3131,7 +3116,7 @@
         <v>5</v>
       </c>
       <c r="M37" s="60" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="N37" s="62"/>
       <c r="O37" s="63">
@@ -3150,25 +3135,25 @@
         <v>18</v>
       </c>
       <c r="D38" s="36" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E38" s="37" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F38" s="36" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G38" s="37" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="H38" s="36" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I38" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J38" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="K38" s="36">
         <v>1</v>
@@ -3178,7 +3163,7 @@
         <v>5</v>
       </c>
       <c r="M38" s="59" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="N38" s="61">
         <v>0.95</v>
@@ -3199,22 +3184,22 @@
         <v>18</v>
       </c>
       <c r="D39" s="38" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E39" s="39" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F39" s="38" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G39" s="39" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H39" s="38" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I39" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J39" s="38"/>
       <c r="K39" s="38">
@@ -3225,7 +3210,7 @@
         <v>5</v>
       </c>
       <c r="M39" s="59" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="N39" s="62"/>
       <c r="O39" s="63">
@@ -3244,25 +3229,25 @@
         <v>19</v>
       </c>
       <c r="D40" s="36" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E40" s="37" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F40" s="36" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G40" s="37" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H40" s="36" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I40" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J40" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="K40" s="36">
         <v>1</v>
@@ -3272,7 +3257,7 @@
         <v>5</v>
       </c>
       <c r="M40" s="60" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="N40" s="61"/>
       <c r="O40" s="63">
@@ -3291,25 +3276,25 @@
         <v>18</v>
       </c>
       <c r="D41" s="38" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E41" s="39" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F41" s="38" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G41" s="39" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="H41" s="38" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="I41" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J41" s="38" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="K41" s="38">
         <v>1</v>
@@ -3319,7 +3304,7 @@
         <v>5</v>
       </c>
       <c r="M41" s="59" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="N41" s="62">
         <v>1.08</v>
@@ -3332,28 +3317,28 @@
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
-      <c r="B42" s="71">
+      <c r="B42" s="66">
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="C42" s="57" t="s">
+        <v>177</v>
+      </c>
+      <c r="D42" s="38" t="s">
+        <v>167</v>
+      </c>
+      <c r="E42" s="38" t="s">
+        <v>167</v>
+      </c>
+      <c r="F42" s="38" t="s">
+        <v>167</v>
+      </c>
+      <c r="G42" s="38" t="s">
         <v>178</v>
-      </c>
-      <c r="D42" s="38" t="s">
-        <v>168</v>
-      </c>
-      <c r="E42" s="38" t="s">
-        <v>168</v>
-      </c>
-      <c r="F42" s="38" t="s">
-        <v>168</v>
-      </c>
-      <c r="G42" s="38" t="s">
-        <v>179</v>
       </c>
       <c r="H42" s="38"/>
       <c r="I42" s="36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J42" s="38"/>
       <c r="K42" s="38">
@@ -3364,7 +3349,7 @@
         <v>5</v>
       </c>
       <c r="M42" s="59" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="N42" s="62">
         <v>0.8</v>
@@ -3377,28 +3362,28 @@
     </row>
     <row r="43" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
-      <c r="B43" s="71">
+      <c r="B43" s="66">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
       <c r="C43" s="57" t="s">
-        <v>178</v>
-      </c>
-      <c r="D43" s="64"/>
-      <c r="E43" s="64"/>
-      <c r="F43" s="64"/>
-      <c r="G43" s="64"/>
-      <c r="H43" s="64"/>
+        <v>177</v>
+      </c>
+      <c r="D43" s="38"/>
+      <c r="E43" s="38"/>
+      <c r="F43" s="38"/>
+      <c r="G43" s="38"/>
+      <c r="H43" s="38"/>
       <c r="I43" s="36" t="s">
-        <v>168</v>
-      </c>
-      <c r="J43" s="64"/>
-      <c r="K43" s="64"/>
-      <c r="L43" s="64"/>
-      <c r="M43" s="65"/>
-      <c r="N43" s="66"/>
-      <c r="O43" s="67"/>
-      <c r="P43" s="68"/>
+        <v>167</v>
+      </c>
+      <c r="J43" s="38"/>
+      <c r="K43" s="38"/>
+      <c r="L43" s="38"/>
+      <c r="M43" s="59"/>
+      <c r="N43" s="62"/>
+      <c r="O43" s="63"/>
+      <c r="P43" s="38"/>
     </row>
     <row r="44" spans="1:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1"/>
@@ -3412,14 +3397,14 @@
       <c r="I44" s="35"/>
       <c r="J44" s="35"/>
       <c r="K44" s="35"/>
-      <c r="L44" s="75" t="s">
-        <v>176</v>
-      </c>
-      <c r="M44" s="76"/>
-      <c r="N44" s="76"/>
-      <c r="O44" s="69">
+      <c r="L44" s="70" t="s">
+        <v>175</v>
+      </c>
+      <c r="M44" s="71"/>
+      <c r="N44" s="71"/>
+      <c r="O44" s="64">
         <f>SUM(O10:O43)</f>
-        <v>44.999999999999993</v>
+        <v>43.999999999999993</v>
       </c>
       <c r="P44" s="41"/>
     </row>
@@ -3435,14 +3420,14 @@
       <c r="I45" s="9"/>
       <c r="J45" s="9"/>
       <c r="K45" s="9"/>
-      <c r="L45" s="75" t="s">
-        <v>177</v>
-      </c>
-      <c r="M45" s="76"/>
-      <c r="N45" s="76"/>
-      <c r="O45" s="70">
+      <c r="L45" s="70" t="s">
+        <v>176</v>
+      </c>
+      <c r="M45" s="71"/>
+      <c r="N45" s="71"/>
+      <c r="O45" s="65">
         <f>O44/5</f>
-        <v>8.9999999999999982</v>
+        <v>8.7999999999999989</v>
       </c>
       <c r="P45" s="42"/>
     </row>

</xml_diff>

<commit_message>
#16 eSpark and Client BOM updates acc to design.
</commit_message>
<xml_diff>
--- a/Design Files/LTE-Module-v2.0/BOM/Client_BOM_v2.0.xlsx
+++ b/Design Files/LTE-Module-v2.0/BOM/Client_BOM_v2.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="179">
   <si>
     <t>Component list</t>
   </si>
@@ -42,9 +42,6 @@
     <t>Item Type</t>
   </si>
   <si>
-    <t>GNSS Antenna</t>
-  </si>
-  <si>
     <t>Capacitor</t>
   </si>
   <si>
@@ -63,9 +60,6 @@
     <t>SIM Card Connectors</t>
   </si>
   <si>
-    <t>Inductor</t>
-  </si>
-  <si>
     <t>LED</t>
   </si>
   <si>
@@ -84,9 +78,6 @@
     <t>Designator</t>
   </si>
   <si>
-    <t>Ant1</t>
-  </si>
-  <si>
     <t>C1</t>
   </si>
   <si>
@@ -129,12 +120,6 @@
     <t>J3</t>
   </si>
   <si>
-    <t>J4</t>
-  </si>
-  <si>
-    <t>L1</t>
-  </si>
-  <si>
     <t>LED1</t>
   </si>
   <si>
@@ -144,9 +129,6 @@
     <t>Q1, Q2, Q3, Q4</t>
   </si>
   <si>
-    <t>R1, R2, R4</t>
-  </si>
-  <si>
     <t>R3, R5</t>
   </si>
   <si>
@@ -165,24 +147,12 @@
     <t>U2</t>
   </si>
   <si>
-    <t>U3</t>
-  </si>
-  <si>
-    <t>U4</t>
-  </si>
-  <si>
     <t>U5</t>
   </si>
   <si>
     <t>Description</t>
   </si>
   <si>
-    <t>1.584GHz GNSS Chip RF Antenna 1.559GHz ~ 1.609GHz 3.1dBi Solder Surface Mount</t>
-  </si>
-  <si>
-    <t>50V 4.3pF C0G 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
-  </si>
-  <si>
     <t>CAP CER 33PF 25V C0G/NP0 0402</t>
   </si>
   <si>
@@ -222,9 +192,6 @@
     <t>Copper Alloy Self bomb Gold plating 1.25mm Deck -40℃~+85℃ 260℃ NanoSIM SMD SIM Card Connectors ROHS</t>
   </si>
   <si>
-    <t>2nH ±0.3nH 0603 Inductors (SMD) ROHS</t>
-  </si>
-  <si>
     <t>Yellow-Green 572nm LED Indication - Discrete 2.05V 0603 (1608 Metric)</t>
   </si>
   <si>
@@ -258,9 +225,6 @@
     <t>IC SWITCH 4PDT 16MLP</t>
   </si>
   <si>
-    <t>GLOBAL IOT EMBEDDED SIM CHIP</t>
-  </si>
-  <si>
     <t>15V 5 Unidirectional 5V SOT-363 ESD Protection Devices ROHS</t>
   </si>
   <si>
@@ -297,9 +261,6 @@
     <t>XKNANO-113</t>
   </si>
   <si>
-    <t>IND-0603 (1608 Metric)</t>
-  </si>
-  <si>
     <t>LED-0603</t>
   </si>
   <si>
@@ -315,9 +276,6 @@
     <t>16-MLP (3x3)</t>
   </si>
   <si>
-    <t>QNF8 (6 x 5mm)</t>
-  </si>
-  <si>
     <t>SOT-363</t>
   </si>
   <si>
@@ -327,12 +285,6 @@
     <t>Manufacturer Part Number</t>
   </si>
   <si>
-    <t>SZC-C-1G18</t>
-  </si>
-  <si>
-    <t>0603CG4R3C500NT</t>
-  </si>
-  <si>
     <t>GRM1555C1E330JA01D</t>
   </si>
   <si>
@@ -366,9 +318,6 @@
     <t>POGO Connector 4 Pin</t>
   </si>
   <si>
-    <t>VHF160808H2N0ST</t>
-  </si>
-  <si>
     <t>19-21/G6C-FM1N2B/3T</t>
   </si>
   <si>
@@ -399,9 +348,6 @@
     <t>FSA2567MPX</t>
   </si>
   <si>
-    <t>SIM-ST-MFF2</t>
-  </si>
-  <si>
     <t>SMF05CT1G-ES</t>
   </si>
   <si>
@@ -411,12 +357,6 @@
     <t>Manufacturer</t>
   </si>
   <si>
-    <t>Synzen</t>
-  </si>
-  <si>
-    <t>FH</t>
-  </si>
-  <si>
     <t>Murata</t>
   </si>
   <si>
@@ -456,21 +396,12 @@
     <t>ON Semiconductor / Fairchild</t>
   </si>
   <si>
-    <t>Hologram</t>
-  </si>
-  <si>
     <t>ElecSuper</t>
   </si>
   <si>
     <t>Texas Instruments</t>
   </si>
   <si>
-    <t>1.559GHz ~ 1.609GHz</t>
-  </si>
-  <si>
-    <t>4.3pF</t>
-  </si>
-  <si>
     <t>33pF</t>
   </si>
   <si>
@@ -489,9 +420,6 @@
     <t>100nF</t>
   </si>
   <si>
-    <t>2nH</t>
-  </si>
-  <si>
     <t>0R</t>
   </si>
   <si>
@@ -585,9 +513,6 @@
     <t>Kyocera AVX</t>
   </si>
   <si>
-    <t>R12, R15, R16, R19, R20</t>
-  </si>
-  <si>
     <t>Bill of Materials for Project [LTE_MODULE_v2.0.]</t>
   </si>
   <si>
@@ -595,6 +520,42 @@
   </si>
   <si>
     <t>C5, C11, C13, C15, C16, C17</t>
+  </si>
+  <si>
+    <t>Antenna</t>
+  </si>
+  <si>
+    <t>ANT1</t>
+  </si>
+  <si>
+    <t>RF ANT 1.575GHZ CHIP SOLDER SMD</t>
+  </si>
+  <si>
+    <t>W3011</t>
+  </si>
+  <si>
+    <t>Pulse</t>
+  </si>
+  <si>
+    <t>CAP CER 2.2PF 50V C0G/NPO 0603</t>
+  </si>
+  <si>
+    <t>CC0603CRNPO9BN2R2</t>
+  </si>
+  <si>
+    <t>2.2pF</t>
+  </si>
+  <si>
+    <t>J4, J5</t>
+  </si>
+  <si>
+    <t>R1, R2, R12, R15, R16, R19, R20</t>
+  </si>
+  <si>
+    <t>R4</t>
+  </si>
+  <si>
+    <t>U3,U4</t>
   </si>
 </sst>
 </file>
@@ -1551,7 +1512,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:P45"/>
+  <dimension ref="A1:P43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="25" customWidth="1"/>
@@ -1598,7 +1559,7 @@
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="51" t="s">
-        <v>189</v>
+        <v>164</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="3"/>
@@ -1620,7 +1581,7 @@
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="52" t="s">
-        <v>190</v>
+        <v>165</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="4"/>
@@ -1642,7 +1603,7 @@
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="53" t="s">
-        <v>190</v>
+        <v>165</v>
       </c>
       <c r="G4" s="13"/>
       <c r="H4" s="6"/>
@@ -1740,74 +1701,74 @@
         <v>6</v>
       </c>
       <c r="D9" s="29" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E9" s="30" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="F9" s="29" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="G9" s="30" t="s">
-        <v>101</v>
+        <v>87</v>
       </c>
       <c r="H9" s="29" t="s">
-        <v>129</v>
+        <v>111</v>
       </c>
       <c r="I9" s="29" t="s">
-        <v>164</v>
+        <v>140</v>
       </c>
       <c r="J9" s="29" t="s">
-        <v>166</v>
+        <v>142</v>
       </c>
       <c r="K9" s="29" t="s">
-        <v>163</v>
+        <v>139</v>
       </c>
       <c r="L9" s="29" t="s">
-        <v>165</v>
+        <v>141</v>
       </c>
       <c r="M9" s="29" t="s">
-        <v>171</v>
+        <v>147</v>
       </c>
       <c r="N9" s="29" t="s">
-        <v>173</v>
+        <v>149</v>
       </c>
       <c r="O9" s="29" t="s">
-        <v>174</v>
+        <v>150</v>
       </c>
       <c r="P9" s="29" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="50">
         <f>ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
       <c r="C10" s="56" t="s">
-        <v>7</v>
+        <v>167</v>
       </c>
       <c r="D10" s="36" t="s">
-        <v>21</v>
-      </c>
-      <c r="E10" s="37" t="s">
-        <v>52</v>
+        <v>168</v>
+      </c>
+      <c r="E10" s="36" t="s">
+        <v>169</v>
       </c>
       <c r="F10" s="36" t="s">
-        <v>168</v>
-      </c>
-      <c r="G10" s="37" t="s">
-        <v>102</v>
+        <v>144</v>
+      </c>
+      <c r="G10" s="36" t="s">
+        <v>170</v>
       </c>
       <c r="H10" s="36" t="s">
-        <v>130</v>
+        <v>171</v>
       </c>
       <c r="I10" s="36" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="J10" s="36" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="K10" s="36">
         <v>1</v>
@@ -1817,46 +1778,46 @@
         <v>5</v>
       </c>
       <c r="M10" s="59" t="s">
-        <v>172</v>
+        <v>148</v>
       </c>
       <c r="N10" s="61">
-        <v>0.9</v>
+        <v>1.59</v>
       </c>
       <c r="O10" s="61">
         <f>N10*L10</f>
-        <v>4.5</v>
+        <v>7.95</v>
       </c>
       <c r="P10" s="36"/>
     </row>
-    <row r="11" spans="1:16" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="50">
-        <f t="shared" ref="B11:B43" si="0">ROW(B11) - ROW($B$9)</f>
+        <f t="shared" ref="B11:B41" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="57" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D11" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="E11" s="39" t="s">
-        <v>53</v>
+        <v>19</v>
+      </c>
+      <c r="E11" s="38" t="s">
+        <v>172</v>
       </c>
       <c r="F11" s="38" t="s">
-        <v>83</v>
-      </c>
-      <c r="G11" s="39" t="s">
-        <v>103</v>
+        <v>71</v>
+      </c>
+      <c r="G11" s="38" t="s">
+        <v>173</v>
       </c>
       <c r="H11" s="38" t="s">
-        <v>131</v>
+        <v>113</v>
       </c>
       <c r="I11" s="36" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="J11" s="38" t="s">
-        <v>149</v>
+        <v>174</v>
       </c>
       <c r="K11" s="38">
         <v>1</v>
@@ -1866,12 +1827,14 @@
         <v>5</v>
       </c>
       <c r="M11" s="60" t="s">
-        <v>180</v>
-      </c>
-      <c r="N11" s="62"/>
+        <v>148</v>
+      </c>
+      <c r="N11" s="62">
+        <v>0.1</v>
+      </c>
       <c r="O11" s="61">
-        <f t="shared" ref="O11:O30" si="2">N11*L11</f>
-        <v>0</v>
+        <f t="shared" ref="O11:O29" si="2">N11*L11</f>
+        <v>0.5</v>
       </c>
       <c r="P11" s="38"/>
     </row>
@@ -1882,28 +1845,28 @@
         <v>3</v>
       </c>
       <c r="C12" s="57" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D12" s="36" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E12" s="37" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="F12" s="36" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="G12" s="37" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="H12" s="36" t="s">
-        <v>132</v>
+        <v>112</v>
       </c>
       <c r="I12" s="36" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="J12" s="36" t="s">
-        <v>150</v>
+        <v>127</v>
       </c>
       <c r="K12" s="36">
         <v>1</v>
@@ -1913,7 +1876,7 @@
         <v>5</v>
       </c>
       <c r="M12" s="59" t="s">
-        <v>172</v>
+        <v>148</v>
       </c>
       <c r="N12" s="61">
         <v>0.1</v>
@@ -1931,28 +1894,28 @@
         <v>4</v>
       </c>
       <c r="C13" s="57" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D13" s="38" t="s">
-        <v>191</v>
+        <v>166</v>
       </c>
       <c r="E13" s="39" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="F13" s="38" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="G13" s="39" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="H13" s="38" t="s">
-        <v>133</v>
+        <v>113</v>
       </c>
       <c r="I13" s="36" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="J13" s="38" t="s">
-        <v>151</v>
+        <v>128</v>
       </c>
       <c r="K13" s="38">
         <v>6</v>
@@ -1962,7 +1925,7 @@
         <v>30</v>
       </c>
       <c r="M13" s="60" t="s">
-        <v>172</v>
+        <v>148</v>
       </c>
       <c r="N13" s="62">
         <v>0.1</v>
@@ -1980,28 +1943,28 @@
         <v>5</v>
       </c>
       <c r="C14" s="56" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D14" s="36" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="E14" s="36" t="s">
-        <v>184</v>
+        <v>160</v>
       </c>
       <c r="F14" s="36" t="s">
-        <v>185</v>
+        <v>161</v>
       </c>
       <c r="G14" s="36" t="s">
-        <v>186</v>
+        <v>162</v>
       </c>
       <c r="H14" s="36" t="s">
-        <v>187</v>
+        <v>163</v>
       </c>
       <c r="I14" s="36" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="J14" s="36" t="s">
-        <v>152</v>
+        <v>129</v>
       </c>
       <c r="K14" s="36">
         <v>1</v>
@@ -2011,7 +1974,7 @@
         <v>5</v>
       </c>
       <c r="M14" s="60" t="s">
-        <v>172</v>
+        <v>148</v>
       </c>
       <c r="N14" s="61">
         <v>1.04</v>
@@ -2029,28 +1992,28 @@
         <v>6</v>
       </c>
       <c r="C15" s="56" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D15" s="38" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E15" s="39" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="F15" s="38" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="G15" s="39" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="H15" s="38" t="s">
-        <v>133</v>
+        <v>113</v>
       </c>
       <c r="I15" s="36" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="J15" s="38" t="s">
-        <v>153</v>
+        <v>130</v>
       </c>
       <c r="K15" s="38">
         <v>1</v>
@@ -2060,7 +2023,7 @@
         <v>5</v>
       </c>
       <c r="M15" s="60" t="s">
-        <v>172</v>
+        <v>148</v>
       </c>
       <c r="N15" s="62">
         <v>0.1</v>
@@ -2078,28 +2041,28 @@
         <v>7</v>
       </c>
       <c r="C16" s="56" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D16" s="36" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E16" s="37" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="F16" s="36" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="G16" s="37" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="H16" s="36" t="s">
-        <v>133</v>
+        <v>113</v>
       </c>
       <c r="I16" s="36" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="J16" s="36" t="s">
-        <v>154</v>
+        <v>131</v>
       </c>
       <c r="K16" s="36">
         <v>3</v>
@@ -2109,7 +2072,7 @@
         <v>15</v>
       </c>
       <c r="M16" s="59" t="s">
-        <v>172</v>
+        <v>148</v>
       </c>
       <c r="N16" s="61">
         <v>0.1</v>
@@ -2127,28 +2090,28 @@
         <v>8</v>
       </c>
       <c r="C17" s="57" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D17" s="38" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E17" s="39" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="F17" s="38" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="G17" s="39" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="H17" s="38" t="s">
-        <v>134</v>
+        <v>114</v>
       </c>
       <c r="I17" s="36" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="J17" s="38" t="s">
-        <v>155</v>
+        <v>132</v>
       </c>
       <c r="K17" s="38">
         <v>2</v>
@@ -2158,7 +2121,7 @@
         <v>10</v>
       </c>
       <c r="M17" s="59" t="s">
-        <v>172</v>
+        <v>148</v>
       </c>
       <c r="N17" s="62">
         <v>0.11</v>
@@ -2176,28 +2139,28 @@
         <v>9</v>
       </c>
       <c r="C18" s="56" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D18" s="36" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E18" s="37" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="F18" s="36" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="G18" s="37" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="H18" s="36" t="s">
-        <v>135</v>
+        <v>115</v>
       </c>
       <c r="I18" s="36" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="J18" s="36" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="K18" s="36">
         <v>1</v>
@@ -2207,7 +2170,7 @@
         <v>5</v>
       </c>
       <c r="M18" s="59" t="s">
-        <v>172</v>
+        <v>148</v>
       </c>
       <c r="N18" s="61">
         <v>0.23</v>
@@ -2225,28 +2188,28 @@
         <v>10</v>
       </c>
       <c r="C19" s="57" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D19" s="38" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E19" s="39" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F19" s="38" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="G19" s="39" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="H19" s="38" t="s">
-        <v>136</v>
+        <v>116</v>
       </c>
       <c r="I19" s="36" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="J19" s="38" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="K19" s="38">
         <v>2</v>
@@ -2256,7 +2219,7 @@
         <v>10</v>
       </c>
       <c r="M19" s="60" t="s">
-        <v>180</v>
+        <v>156</v>
       </c>
       <c r="N19" s="62"/>
       <c r="O19" s="61">
@@ -2272,28 +2235,28 @@
         <v>11</v>
       </c>
       <c r="C20" s="56" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D20" s="36" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E20" s="37" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="F20" s="36" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="G20" s="37" t="s">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="H20" s="36" t="s">
-        <v>137</v>
+        <v>117</v>
       </c>
       <c r="I20" s="36" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="J20" s="36" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="K20" s="36">
         <v>1</v>
@@ -2303,7 +2266,7 @@
         <v>5</v>
       </c>
       <c r="M20" s="59" t="s">
-        <v>172</v>
+        <v>148</v>
       </c>
       <c r="N20" s="61">
         <v>0.48</v>
@@ -2321,28 +2284,28 @@
         <v>12</v>
       </c>
       <c r="C21" s="57" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D21" s="38" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E21" s="39" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="F21" s="38" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="G21" s="39" t="s">
-        <v>112</v>
+        <v>96</v>
       </c>
       <c r="H21" s="38" t="s">
-        <v>138</v>
+        <v>118</v>
       </c>
       <c r="I21" s="36" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="J21" s="38" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="K21" s="38">
         <v>1</v>
@@ -2352,7 +2315,7 @@
         <v>5</v>
       </c>
       <c r="M21" s="60" t="s">
-        <v>180</v>
+        <v>156</v>
       </c>
       <c r="N21" s="62"/>
       <c r="O21" s="61">
@@ -2368,28 +2331,28 @@
         <v>13</v>
       </c>
       <c r="C22" s="56" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D22" s="36" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E22" s="37" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="F22" s="36" t="s">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="G22" s="37" t="s">
-        <v>113</v>
+        <v>97</v>
       </c>
       <c r="H22" s="36" t="s">
-        <v>139</v>
+        <v>119</v>
       </c>
       <c r="I22" s="36" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="J22" s="36" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="K22" s="36">
         <v>1</v>
@@ -2399,7 +2362,7 @@
         <v>5</v>
       </c>
       <c r="M22" s="60" t="s">
-        <v>180</v>
+        <v>156</v>
       </c>
       <c r="N22" s="61"/>
       <c r="O22" s="61">
@@ -2415,28 +2378,28 @@
         <v>14</v>
       </c>
       <c r="C23" s="57" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D23" s="38" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E23" s="38" t="s">
-        <v>181</v>
+        <v>157</v>
       </c>
       <c r="F23" s="38" t="s">
-        <v>168</v>
+        <v>144</v>
       </c>
       <c r="G23" s="38" t="s">
-        <v>182</v>
+        <v>158</v>
       </c>
       <c r="H23" s="38" t="s">
-        <v>183</v>
+        <v>159</v>
       </c>
       <c r="I23" s="36" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="J23" s="38" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="K23" s="38">
         <v>1</v>
@@ -2446,7 +2409,7 @@
         <v>5</v>
       </c>
       <c r="M23" s="60" t="s">
-        <v>180</v>
+        <v>156</v>
       </c>
       <c r="N23" s="62"/>
       <c r="O23" s="61">
@@ -2462,28 +2425,28 @@
         <v>15</v>
       </c>
       <c r="C24" s="56" t="s">
-        <v>169</v>
+        <v>145</v>
       </c>
       <c r="D24" s="36" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="E24" s="37" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="F24" s="55" t="s">
-        <v>168</v>
+        <v>144</v>
       </c>
       <c r="G24" s="37" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="H24" s="36" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="I24" s="36" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="J24" s="55" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="K24" s="36">
         <v>1</v>
@@ -2493,7 +2456,7 @@
         <v>5</v>
       </c>
       <c r="M24" s="55" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="N24" s="61"/>
       <c r="O24" s="61">
@@ -2509,28 +2472,28 @@
         <v>16</v>
       </c>
       <c r="C25" s="57" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D25" s="38" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E25" s="39" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="F25" s="38" t="s">
-        <v>168</v>
+        <v>144</v>
       </c>
       <c r="G25" s="39" t="s">
-        <v>114</v>
+        <v>98</v>
       </c>
       <c r="H25" s="36" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="I25" s="36" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="J25" s="55" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="K25" s="38">
         <v>1</v>
@@ -2540,7 +2503,7 @@
         <v>5</v>
       </c>
       <c r="M25" s="55" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="N25" s="62"/>
       <c r="O25" s="61">
@@ -2556,38 +2519,38 @@
         <v>17</v>
       </c>
       <c r="C26" s="56" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D26" s="36" t="s">
-        <v>36</v>
+        <v>175</v>
       </c>
       <c r="E26" s="37" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="F26" s="36" t="s">
-        <v>168</v>
+        <v>144</v>
       </c>
       <c r="G26" s="37" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="H26" s="36" t="s">
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="I26" s="36" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="J26" s="36" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="K26" s="36">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L26" s="36">
         <f>K26*5</f>
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="M26" s="60" t="s">
-        <v>180</v>
+        <v>156</v>
       </c>
       <c r="N26" s="61"/>
       <c r="O26" s="61">
@@ -2599,288 +2562,290 @@
     <row r="27" spans="1:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B27) - ROW($B$9)</f>
         <v>18</v>
       </c>
-      <c r="C27" s="57" t="s">
-        <v>14</v>
-      </c>
-      <c r="D27" s="38" t="s">
-        <v>37</v>
-      </c>
-      <c r="E27" s="39" t="s">
-        <v>67</v>
-      </c>
-      <c r="F27" s="38" t="s">
-        <v>92</v>
-      </c>
-      <c r="G27" s="39" t="s">
-        <v>115</v>
-      </c>
-      <c r="H27" s="38" t="s">
-        <v>131</v>
+      <c r="C27" s="56" t="s">
+        <v>13</v>
+      </c>
+      <c r="D27" s="36" t="s">
+        <v>33</v>
+      </c>
+      <c r="E27" s="37" t="s">
+        <v>57</v>
+      </c>
+      <c r="F27" s="36" t="s">
+        <v>80</v>
+      </c>
+      <c r="G27" s="37" t="s">
+        <v>99</v>
+      </c>
+      <c r="H27" s="36" t="s">
+        <v>121</v>
       </c>
       <c r="I27" s="36" t="s">
-        <v>167</v>
-      </c>
-      <c r="J27" s="38" t="s">
+        <v>143</v>
+      </c>
+      <c r="J27" s="36" t="s">
+        <v>143</v>
+      </c>
+      <c r="K27" s="36">
+        <v>1</v>
+      </c>
+      <c r="L27" s="36">
+        <f>K27*5</f>
+        <v>5</v>
+      </c>
+      <c r="M27" s="60" t="s">
         <v>156</v>
       </c>
-      <c r="K27" s="38">
-        <v>1</v>
-      </c>
-      <c r="L27" s="38">
-        <f t="shared" ref="L27" si="10">K27*5</f>
-        <v>5</v>
-      </c>
-      <c r="M27" s="60" t="s">
-        <v>180</v>
-      </c>
-      <c r="N27" s="62"/>
+      <c r="N27" s="61"/>
       <c r="O27" s="61">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="P27" s="38"/>
+      <c r="P27" s="36"/>
     </row>
     <row r="28" spans="1:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="50">
-        <f>ROW(B28) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="C28" s="56" t="s">
-        <v>15</v>
-      </c>
-      <c r="D28" s="36" t="s">
-        <v>38</v>
-      </c>
-      <c r="E28" s="37" t="s">
-        <v>68</v>
-      </c>
-      <c r="F28" s="36" t="s">
-        <v>93</v>
-      </c>
-      <c r="G28" s="37" t="s">
-        <v>116</v>
-      </c>
-      <c r="H28" s="36" t="s">
-        <v>141</v>
+      <c r="C28" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="D28" s="38" t="s">
+        <v>34</v>
+      </c>
+      <c r="E28" s="39" t="s">
+        <v>58</v>
+      </c>
+      <c r="F28" s="38" t="s">
+        <v>80</v>
+      </c>
+      <c r="G28" s="39" t="s">
+        <v>100</v>
+      </c>
+      <c r="H28" s="38" t="s">
+        <v>121</v>
       </c>
       <c r="I28" s="36" t="s">
-        <v>167</v>
-      </c>
-      <c r="J28" s="36" t="s">
-        <v>167</v>
-      </c>
-      <c r="K28" s="36">
+        <v>143</v>
+      </c>
+      <c r="J28" s="38" t="s">
+        <v>143</v>
+      </c>
+      <c r="K28" s="38">
         <v>1</v>
       </c>
-      <c r="L28" s="36">
-        <f>K28*5</f>
+      <c r="L28" s="38">
+        <f t="shared" ref="L28" si="10">K28*5</f>
         <v>5</v>
       </c>
       <c r="M28" s="60" t="s">
-        <v>180</v>
-      </c>
-      <c r="N28" s="61"/>
+        <v>156</v>
+      </c>
+      <c r="N28" s="62"/>
       <c r="O28" s="61">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="P28" s="36"/>
-    </row>
-    <row r="29" spans="1:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P28" s="38"/>
+    </row>
+    <row r="29" spans="1:16" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B29) - ROW($B$9)</f>
         <v>20</v>
       </c>
-      <c r="C29" s="57" t="s">
-        <v>15</v>
-      </c>
-      <c r="D29" s="38" t="s">
-        <v>39</v>
-      </c>
-      <c r="E29" s="39" t="s">
-        <v>69</v>
-      </c>
-      <c r="F29" s="38" t="s">
-        <v>93</v>
-      </c>
-      <c r="G29" s="39" t="s">
-        <v>117</v>
-      </c>
-      <c r="H29" s="38" t="s">
-        <v>141</v>
+      <c r="C29" s="56" t="s">
+        <v>14</v>
+      </c>
+      <c r="D29" s="36" t="s">
+        <v>35</v>
+      </c>
+      <c r="E29" s="37" t="s">
+        <v>59</v>
+      </c>
+      <c r="F29" s="36" t="s">
+        <v>81</v>
+      </c>
+      <c r="G29" s="37" t="s">
+        <v>101</v>
+      </c>
+      <c r="H29" s="36" t="s">
+        <v>122</v>
       </c>
       <c r="I29" s="36" t="s">
-        <v>167</v>
-      </c>
-      <c r="J29" s="38" t="s">
-        <v>167</v>
-      </c>
-      <c r="K29" s="38">
-        <v>1</v>
-      </c>
-      <c r="L29" s="38">
-        <f t="shared" ref="L29" si="11">K29*5</f>
-        <v>5</v>
+        <v>143</v>
+      </c>
+      <c r="J29" s="36" t="s">
+        <v>143</v>
+      </c>
+      <c r="K29" s="36">
+        <v>4</v>
+      </c>
+      <c r="L29" s="36">
+        <f>K29*5</f>
+        <v>20</v>
       </c>
       <c r="M29" s="60" t="s">
-        <v>180</v>
-      </c>
-      <c r="N29" s="62"/>
+        <v>156</v>
+      </c>
+      <c r="N29" s="61"/>
       <c r="O29" s="61">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="P29" s="38"/>
-    </row>
-    <row r="30" spans="1:16" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P29" s="36"/>
+    </row>
+    <row r="30" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="50">
         <f>ROW(B30) - ROW($B$9)</f>
         <v>21</v>
       </c>
       <c r="C30" s="56" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D30" s="36" t="s">
-        <v>40</v>
+        <v>176</v>
       </c>
       <c r="E30" s="37" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="F30" s="36" t="s">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="G30" s="37" t="s">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="H30" s="36" t="s">
-        <v>142</v>
+        <v>113</v>
       </c>
       <c r="I30" s="36" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="J30" s="36" t="s">
-        <v>167</v>
+        <v>138</v>
       </c>
       <c r="K30" s="36">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L30" s="36">
         <f>K30*5</f>
-        <v>20</v>
-      </c>
-      <c r="M30" s="60" t="s">
-        <v>180</v>
-      </c>
-      <c r="N30" s="61"/>
-      <c r="O30" s="61">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <v>35</v>
+      </c>
+      <c r="M30" s="59" t="s">
+        <v>148</v>
+      </c>
+      <c r="N30" s="62">
+        <v>0.1</v>
+      </c>
+      <c r="O30" s="63">
+        <f>N30*L30</f>
+        <v>3.5</v>
       </c>
       <c r="P30" s="36"/>
     </row>
     <row r="31" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B31) - ROW($B$9)</f>
         <v>22</v>
       </c>
-      <c r="C31" s="57" t="s">
-        <v>17</v>
-      </c>
-      <c r="D31" s="38" t="s">
-        <v>41</v>
-      </c>
-      <c r="E31" s="39" t="s">
-        <v>71</v>
-      </c>
-      <c r="F31" s="38" t="s">
-        <v>95</v>
-      </c>
-      <c r="G31" s="39" t="s">
-        <v>119</v>
-      </c>
-      <c r="H31" s="38" t="s">
-        <v>133</v>
+      <c r="C31" s="56" t="s">
+        <v>15</v>
+      </c>
+      <c r="D31" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="E31" s="37" t="s">
+        <v>61</v>
+      </c>
+      <c r="F31" s="36" t="s">
+        <v>82</v>
+      </c>
+      <c r="G31" s="37" t="s">
+        <v>103</v>
+      </c>
+      <c r="H31" s="36" t="s">
+        <v>113</v>
       </c>
       <c r="I31" s="36" t="s">
-        <v>167</v>
-      </c>
-      <c r="J31" s="38" t="s">
-        <v>157</v>
-      </c>
-      <c r="K31" s="38">
-        <v>3</v>
-      </c>
-      <c r="L31" s="38">
-        <f t="shared" ref="L31" si="12">K31*5</f>
-        <v>15</v>
+        <v>143</v>
+      </c>
+      <c r="J31" s="36" t="s">
+        <v>134</v>
+      </c>
+      <c r="K31" s="36">
+        <v>2</v>
+      </c>
+      <c r="L31" s="36">
+        <f>K31*5</f>
+        <v>10</v>
       </c>
       <c r="M31" s="59" t="s">
-        <v>172</v>
+        <v>148</v>
       </c>
       <c r="N31" s="62">
         <v>0.1</v>
       </c>
       <c r="O31" s="63">
         <f>N31*L31</f>
-        <v>1.5</v>
-      </c>
-      <c r="P31" s="38"/>
+        <v>1</v>
+      </c>
+      <c r="P31" s="36"/>
     </row>
     <row r="32" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="50">
-        <f>ROW(B32) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="C32" s="56" t="s">
-        <v>17</v>
-      </c>
-      <c r="D32" s="36" t="s">
-        <v>42</v>
-      </c>
-      <c r="E32" s="37" t="s">
-        <v>72</v>
-      </c>
-      <c r="F32" s="36" t="s">
-        <v>95</v>
-      </c>
-      <c r="G32" s="37" t="s">
-        <v>120</v>
-      </c>
-      <c r="H32" s="36" t="s">
+      <c r="C32" s="57" t="s">
+        <v>15</v>
+      </c>
+      <c r="D32" s="38" t="s">
+        <v>177</v>
+      </c>
+      <c r="E32" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="F32" s="38" t="s">
+        <v>82</v>
+      </c>
+      <c r="G32" s="39" t="s">
+        <v>102</v>
+      </c>
+      <c r="H32" s="38" t="s">
+        <v>113</v>
+      </c>
+      <c r="I32" s="36" t="s">
+        <v>143</v>
+      </c>
+      <c r="J32" s="38" t="s">
         <v>133</v>
       </c>
-      <c r="I32" s="36" t="s">
-        <v>167</v>
-      </c>
-      <c r="J32" s="36" t="s">
-        <v>158</v>
-      </c>
-      <c r="K32" s="36">
-        <v>2</v>
-      </c>
-      <c r="L32" s="36">
-        <f>K32*5</f>
-        <v>10</v>
+      <c r="K32" s="38">
+        <v>1</v>
+      </c>
+      <c r="L32" s="38">
+        <f t="shared" ref="L32" si="11">K32*5</f>
+        <v>5</v>
       </c>
       <c r="M32" s="59" t="s">
-        <v>172</v>
+        <v>148</v>
       </c>
       <c r="N32" s="62">
         <v>0.1</v>
       </c>
       <c r="O32" s="63">
-        <f t="shared" ref="O32:O42" si="13">N32*L32</f>
-        <v>1</v>
-      </c>
-      <c r="P32" s="36"/>
+        <f>N32*L32</f>
+        <v>0.5</v>
+      </c>
+      <c r="P32" s="38"/>
     </row>
     <row r="33" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
@@ -2889,44 +2854,44 @@
         <v>24</v>
       </c>
       <c r="C33" s="57" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D33" s="38" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="E33" s="39" t="s">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="F33" s="38" t="s">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="G33" s="39" t="s">
-        <v>121</v>
+        <v>104</v>
       </c>
       <c r="H33" s="38" t="s">
-        <v>133</v>
+        <v>113</v>
       </c>
       <c r="I33" s="36" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="J33" s="38" t="s">
-        <v>159</v>
+        <v>135</v>
       </c>
       <c r="K33" s="38">
         <v>2</v>
       </c>
       <c r="L33" s="38">
-        <f t="shared" ref="L33" si="14">K33*5</f>
+        <f t="shared" ref="L33" si="12">K33*5</f>
         <v>10</v>
       </c>
       <c r="M33" s="59" t="s">
-        <v>172</v>
+        <v>148</v>
       </c>
       <c r="N33" s="62">
         <v>0.1</v>
       </c>
       <c r="O33" s="63">
-        <f t="shared" si="13"/>
+        <f t="shared" ref="O33:O40" si="13">N33*L33</f>
         <v>1</v>
       </c>
       <c r="P33" s="38"/>
@@ -2938,28 +2903,28 @@
         <v>25</v>
       </c>
       <c r="C34" s="56" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D34" s="36" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="E34" s="37" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="F34" s="36" t="s">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="G34" s="37" t="s">
-        <v>122</v>
+        <v>105</v>
       </c>
       <c r="H34" s="36" t="s">
-        <v>133</v>
+        <v>113</v>
       </c>
       <c r="I34" s="36" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="J34" s="36" t="s">
-        <v>160</v>
+        <v>136</v>
       </c>
       <c r="K34" s="36">
         <v>4</v>
@@ -2969,7 +2934,7 @@
         <v>20</v>
       </c>
       <c r="M34" s="59" t="s">
-        <v>172</v>
+        <v>148</v>
       </c>
       <c r="N34" s="62">
         <v>0.1</v>
@@ -2987,38 +2952,38 @@
         <v>26</v>
       </c>
       <c r="C35" s="56" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D35" s="38" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="E35" s="39" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="F35" s="38" t="s">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="G35" s="39" t="s">
-        <v>123</v>
+        <v>106</v>
       </c>
       <c r="H35" s="38" t="s">
-        <v>133</v>
+        <v>113</v>
       </c>
       <c r="I35" s="36" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="J35" s="38" t="s">
-        <v>161</v>
+        <v>137</v>
       </c>
       <c r="K35" s="38">
         <v>4</v>
       </c>
       <c r="L35" s="38">
-        <f t="shared" ref="L35" si="15">K35*5</f>
+        <f t="shared" ref="L35" si="14">K35*5</f>
         <v>20</v>
       </c>
       <c r="M35" s="59" t="s">
-        <v>172</v>
+        <v>148</v>
       </c>
       <c r="N35" s="62">
         <v>0.1</v>
@@ -3029,131 +2994,131 @@
       </c>
       <c r="P35" s="38"/>
     </row>
-    <row r="36" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="B36" s="50">
-        <f>ROW(B36) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>27</v>
       </c>
-      <c r="C36" s="56" t="s">
-        <v>17</v>
-      </c>
-      <c r="D36" s="36" t="s">
-        <v>188</v>
-      </c>
-      <c r="E36" s="37" t="s">
-        <v>76</v>
-      </c>
-      <c r="F36" s="36" t="s">
-        <v>95</v>
-      </c>
-      <c r="G36" s="37" t="s">
-        <v>124</v>
-      </c>
-      <c r="H36" s="36" t="s">
-        <v>133</v>
+      <c r="C36" s="57" t="s">
+        <v>16</v>
+      </c>
+      <c r="D36" s="38" t="s">
+        <v>40</v>
+      </c>
+      <c r="E36" s="39" t="s">
+        <v>66</v>
+      </c>
+      <c r="F36" s="38" t="s">
+        <v>144</v>
+      </c>
+      <c r="G36" s="39" t="s">
+        <v>83</v>
+      </c>
+      <c r="H36" s="38" t="s">
+        <v>123</v>
       </c>
       <c r="I36" s="36" t="s">
-        <v>167</v>
-      </c>
-      <c r="J36" s="36" t="s">
-        <v>162</v>
-      </c>
-      <c r="K36" s="36">
+        <v>143</v>
+      </c>
+      <c r="J36" s="38" t="s">
+        <v>143</v>
+      </c>
+      <c r="K36" s="38">
+        <v>1</v>
+      </c>
+      <c r="L36" s="38">
+        <f t="shared" ref="L36" si="15">K36*5</f>
         <v>5</v>
       </c>
-      <c r="L36" s="36">
-        <f>K36*5</f>
-        <v>25</v>
-      </c>
-      <c r="M36" s="59" t="s">
-        <v>172</v>
-      </c>
-      <c r="N36" s="62">
-        <v>0.1</v>
-      </c>
+      <c r="M36" s="60" t="s">
+        <v>156</v>
+      </c>
+      <c r="N36" s="62"/>
       <c r="O36" s="63">
         <f t="shared" si="13"/>
-        <v>2.5</v>
-      </c>
-      <c r="P36" s="36"/>
-    </row>
-    <row r="37" spans="1:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+      <c r="P36" s="38"/>
+    </row>
+    <row r="37" spans="1:16" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B37) - ROW($B$9)</f>
         <v>28</v>
       </c>
-      <c r="C37" s="57" t="s">
-        <v>18</v>
-      </c>
-      <c r="D37" s="38" t="s">
-        <v>46</v>
-      </c>
-      <c r="E37" s="39" t="s">
-        <v>77</v>
-      </c>
-      <c r="F37" s="38" t="s">
-        <v>168</v>
-      </c>
-      <c r="G37" s="39" t="s">
-        <v>96</v>
-      </c>
-      <c r="H37" s="38" t="s">
-        <v>143</v>
+      <c r="C37" s="56" t="s">
+        <v>16</v>
+      </c>
+      <c r="D37" s="36" t="s">
+        <v>41</v>
+      </c>
+      <c r="E37" s="37" t="s">
+        <v>67</v>
+      </c>
+      <c r="F37" s="36" t="s">
+        <v>84</v>
+      </c>
+      <c r="G37" s="37" t="s">
+        <v>108</v>
+      </c>
+      <c r="H37" s="36" t="s">
+        <v>124</v>
       </c>
       <c r="I37" s="36" t="s">
-        <v>167</v>
-      </c>
-      <c r="J37" s="38" t="s">
-        <v>167</v>
-      </c>
-      <c r="K37" s="38">
+        <v>143</v>
+      </c>
+      <c r="J37" s="36" t="s">
+        <v>143</v>
+      </c>
+      <c r="K37" s="36">
         <v>1</v>
       </c>
-      <c r="L37" s="38">
-        <f t="shared" ref="L37" si="16">K37*5</f>
+      <c r="L37" s="36">
+        <f>K37*5</f>
         <v>5</v>
       </c>
-      <c r="M37" s="60" t="s">
-        <v>180</v>
-      </c>
-      <c r="N37" s="62"/>
+      <c r="M37" s="59" t="s">
+        <v>148</v>
+      </c>
+      <c r="N37" s="61">
+        <v>0.95</v>
+      </c>
       <c r="O37" s="63">
         <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="P37" s="38"/>
-    </row>
-    <row r="38" spans="1:16" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>4.75</v>
+      </c>
+      <c r="P37" s="36"/>
+    </row>
+    <row r="38" spans="1:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
       <c r="B38" s="50">
         <f>ROW(B38) - ROW($B$9)</f>
         <v>29</v>
       </c>
       <c r="C38" s="56" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D38" s="36" t="s">
-        <v>47</v>
+        <v>178</v>
       </c>
       <c r="E38" s="37" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="F38" s="36" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="G38" s="37" t="s">
+        <v>109</v>
+      </c>
+      <c r="H38" s="36" t="s">
         <v>125</v>
       </c>
-      <c r="H38" s="36" t="s">
-        <v>144</v>
-      </c>
       <c r="I38" s="36" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="J38" s="36" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="K38" s="36">
         <v>1</v>
@@ -3162,15 +3127,13 @@
         <f>K38*5</f>
         <v>5</v>
       </c>
-      <c r="M38" s="59" t="s">
-        <v>172</v>
-      </c>
-      <c r="N38" s="61">
-        <v>0.95</v>
-      </c>
+      <c r="M38" s="60" t="s">
+        <v>156</v>
+      </c>
+      <c r="N38" s="61"/>
       <c r="O38" s="63">
         <f t="shared" si="13"/>
-        <v>4.75</v>
+        <v>0</v>
       </c>
       <c r="P38" s="36"/>
     </row>
@@ -3181,283 +3144,191 @@
         <v>30</v>
       </c>
       <c r="C39" s="57" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D39" s="38" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="E39" s="39" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="F39" s="38" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="G39" s="39" t="s">
+        <v>110</v>
+      </c>
+      <c r="H39" s="38" t="s">
         <v>126</v>
       </c>
-      <c r="H39" s="38" t="s">
-        <v>145</v>
-      </c>
       <c r="I39" s="36" t="s">
-        <v>167</v>
-      </c>
-      <c r="J39" s="38"/>
+        <v>143</v>
+      </c>
+      <c r="J39" s="38" t="s">
+        <v>143</v>
+      </c>
       <c r="K39" s="38">
         <v>1</v>
       </c>
       <c r="L39" s="38">
-        <f t="shared" ref="L39" si="17">K39*5</f>
+        <f t="shared" ref="L39:L40" si="16">K39*5</f>
         <v>5</v>
       </c>
       <c r="M39" s="59" t="s">
-        <v>172</v>
-      </c>
-      <c r="N39" s="62"/>
+        <v>148</v>
+      </c>
+      <c r="N39" s="62">
+        <v>1.08</v>
+      </c>
       <c r="O39" s="63">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>5.4</v>
       </c>
       <c r="P39" s="38"/>
     </row>
-    <row r="40" spans="1:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
-      <c r="B40" s="50">
-        <f>ROW(B40) - ROW($B$9)</f>
+      <c r="B40" s="66">
+        <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="C40" s="56" t="s">
-        <v>19</v>
-      </c>
-      <c r="D40" s="36" t="s">
-        <v>49</v>
-      </c>
-      <c r="E40" s="37" t="s">
-        <v>80</v>
-      </c>
-      <c r="F40" s="36" t="s">
-        <v>99</v>
-      </c>
-      <c r="G40" s="37" t="s">
-        <v>127</v>
-      </c>
-      <c r="H40" s="36" t="s">
-        <v>146</v>
-      </c>
+      <c r="C40" s="57" t="s">
+        <v>153</v>
+      </c>
+      <c r="D40" s="38" t="s">
+        <v>143</v>
+      </c>
+      <c r="E40" s="38" t="s">
+        <v>143</v>
+      </c>
+      <c r="F40" s="38" t="s">
+        <v>143</v>
+      </c>
+      <c r="G40" s="38" t="s">
+        <v>154</v>
+      </c>
+      <c r="H40" s="38"/>
       <c r="I40" s="36" t="s">
-        <v>167</v>
-      </c>
-      <c r="J40" s="36" t="s">
-        <v>167</v>
-      </c>
-      <c r="K40" s="36">
+        <v>143</v>
+      </c>
+      <c r="J40" s="38"/>
+      <c r="K40" s="38">
         <v>1</v>
       </c>
-      <c r="L40" s="36">
-        <f>K40*5</f>
+      <c r="L40" s="38">
+        <f t="shared" si="16"/>
         <v>5</v>
       </c>
-      <c r="M40" s="60" t="s">
-        <v>180</v>
-      </c>
-      <c r="N40" s="61"/>
+      <c r="M40" s="59" t="s">
+        <v>155</v>
+      </c>
+      <c r="N40" s="62">
+        <v>0.8</v>
+      </c>
       <c r="O40" s="63">
         <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="P40" s="36"/>
+        <v>4</v>
+      </c>
+      <c r="P40" s="38"/>
     </row>
     <row r="41" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
-      <c r="B41" s="50">
+      <c r="B41" s="66">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="C41" s="57" t="s">
-        <v>18</v>
-      </c>
-      <c r="D41" s="38" t="s">
-        <v>50</v>
-      </c>
-      <c r="E41" s="39" t="s">
-        <v>81</v>
-      </c>
-      <c r="F41" s="38" t="s">
-        <v>100</v>
-      </c>
-      <c r="G41" s="39" t="s">
-        <v>128</v>
-      </c>
-      <c r="H41" s="38" t="s">
-        <v>147</v>
-      </c>
+        <v>153</v>
+      </c>
+      <c r="D41" s="38"/>
+      <c r="E41" s="38"/>
+      <c r="F41" s="38"/>
+      <c r="G41" s="38"/>
+      <c r="H41" s="38"/>
       <c r="I41" s="36" t="s">
-        <v>167</v>
-      </c>
-      <c r="J41" s="38" t="s">
-        <v>167</v>
-      </c>
-      <c r="K41" s="38">
-        <v>1</v>
-      </c>
-      <c r="L41" s="38">
-        <f t="shared" ref="L41:L42" si="18">K41*5</f>
-        <v>5</v>
-      </c>
-      <c r="M41" s="59" t="s">
-        <v>172</v>
-      </c>
-      <c r="N41" s="62">
-        <v>1.08</v>
-      </c>
-      <c r="O41" s="63">
-        <f t="shared" si="13"/>
-        <v>5.4</v>
-      </c>
+        <v>143</v>
+      </c>
+      <c r="J41" s="38"/>
+      <c r="K41" s="38"/>
+      <c r="L41" s="38"/>
+      <c r="M41" s="59"/>
+      <c r="N41" s="62"/>
+      <c r="O41" s="63"/>
       <c r="P41" s="38"/>
     </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
-      <c r="B42" s="66">
-        <f t="shared" si="0"/>
-        <v>33</v>
-      </c>
-      <c r="C42" s="57" t="s">
-        <v>177</v>
-      </c>
-      <c r="D42" s="38" t="s">
-        <v>167</v>
-      </c>
-      <c r="E42" s="38" t="s">
-        <v>167</v>
-      </c>
-      <c r="F42" s="38" t="s">
-        <v>167</v>
-      </c>
-      <c r="G42" s="38" t="s">
-        <v>178</v>
-      </c>
-      <c r="H42" s="38"/>
-      <c r="I42" s="36" t="s">
-        <v>167</v>
-      </c>
-      <c r="J42" s="38"/>
-      <c r="K42" s="38">
-        <v>1</v>
-      </c>
-      <c r="L42" s="38">
-        <f t="shared" si="18"/>
-        <v>5</v>
-      </c>
-      <c r="M42" s="59" t="s">
-        <v>179</v>
-      </c>
-      <c r="N42" s="62">
-        <v>0.8</v>
-      </c>
-      <c r="O42" s="63">
-        <f t="shared" si="13"/>
-        <v>4</v>
-      </c>
-      <c r="P42" s="38"/>
-    </row>
-    <row r="43" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B42" s="31"/>
+      <c r="C42" s="48"/>
+      <c r="D42" s="32"/>
+      <c r="E42" s="33"/>
+      <c r="F42" s="34"/>
+      <c r="G42" s="35"/>
+      <c r="H42" s="34"/>
+      <c r="I42" s="35"/>
+      <c r="J42" s="35"/>
+      <c r="K42" s="35"/>
+      <c r="L42" s="70" t="s">
+        <v>151</v>
+      </c>
+      <c r="M42" s="71"/>
+      <c r="N42" s="71"/>
+      <c r="O42" s="64">
+        <f>SUM(O10:O41)</f>
+        <v>47.949999999999996</v>
+      </c>
+      <c r="P42" s="41"/>
+    </row>
+    <row r="43" spans="1:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
-      <c r="B43" s="66">
-        <f t="shared" si="0"/>
-        <v>34</v>
-      </c>
-      <c r="C43" s="57" t="s">
-        <v>177</v>
-      </c>
-      <c r="D43" s="38"/>
-      <c r="E43" s="38"/>
-      <c r="F43" s="38"/>
-      <c r="G43" s="38"/>
-      <c r="H43" s="38"/>
-      <c r="I43" s="36" t="s">
-        <v>167</v>
-      </c>
-      <c r="J43" s="38"/>
-      <c r="K43" s="38"/>
-      <c r="L43" s="38"/>
-      <c r="M43" s="59"/>
-      <c r="N43" s="62"/>
-      <c r="O43" s="63"/>
-      <c r="P43" s="38"/>
-    </row>
-    <row r="44" spans="1:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="1"/>
-      <c r="B44" s="31"/>
-      <c r="C44" s="48"/>
-      <c r="D44" s="32"/>
-      <c r="E44" s="33"/>
-      <c r="F44" s="34"/>
-      <c r="G44" s="35"/>
-      <c r="H44" s="34"/>
-      <c r="I44" s="35"/>
-      <c r="J44" s="35"/>
-      <c r="K44" s="35"/>
-      <c r="L44" s="70" t="s">
-        <v>175</v>
-      </c>
-      <c r="M44" s="71"/>
-      <c r="N44" s="71"/>
-      <c r="O44" s="64">
-        <f>SUM(O10:O43)</f>
-        <v>43.999999999999993</v>
-      </c>
-      <c r="P44" s="41"/>
-    </row>
-    <row r="45" spans="1:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="1"/>
-      <c r="B45" s="24"/>
-      <c r="C45" s="49"/>
-      <c r="D45" s="8"/>
-      <c r="E45" s="9"/>
-      <c r="F45" s="9"/>
-      <c r="G45" s="9"/>
-      <c r="H45" s="9"/>
-      <c r="I45" s="9"/>
-      <c r="J45" s="9"/>
-      <c r="K45" s="9"/>
-      <c r="L45" s="70" t="s">
-        <v>176</v>
-      </c>
-      <c r="M45" s="71"/>
-      <c r="N45" s="71"/>
-      <c r="O45" s="65">
-        <f>O44/5</f>
-        <v>8.7999999999999989</v>
-      </c>
-      <c r="P45" s="42"/>
+      <c r="B43" s="24"/>
+      <c r="C43" s="49"/>
+      <c r="D43" s="8"/>
+      <c r="E43" s="9"/>
+      <c r="F43" s="9"/>
+      <c r="G43" s="9"/>
+      <c r="H43" s="9"/>
+      <c r="I43" s="9"/>
+      <c r="J43" s="9"/>
+      <c r="K43" s="9"/>
+      <c r="L43" s="70" t="s">
+        <v>152</v>
+      </c>
+      <c r="M43" s="71"/>
+      <c r="N43" s="71"/>
+      <c r="O43" s="65">
+        <f>O42/5</f>
+        <v>9.59</v>
+      </c>
+      <c r="P43" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="J1:P1"/>
     <mergeCell ref="P3:P8"/>
-    <mergeCell ref="L44:N44"/>
-    <mergeCell ref="L45:N45"/>
+    <mergeCell ref="L42:N42"/>
+    <mergeCell ref="L43:N43"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="M10" r:id="rId1"/>
-    <hyperlink ref="M12" r:id="rId2"/>
-    <hyperlink ref="M13" r:id="rId3"/>
-    <hyperlink ref="M15" r:id="rId4"/>
-    <hyperlink ref="M16" r:id="rId5"/>
-    <hyperlink ref="M17" r:id="rId6"/>
-    <hyperlink ref="M18" r:id="rId7"/>
-    <hyperlink ref="M20" r:id="rId8"/>
+    <hyperlink ref="M12" r:id="rId1"/>
+    <hyperlink ref="M13" r:id="rId2"/>
+    <hyperlink ref="M15" r:id="rId3"/>
+    <hyperlink ref="M16" r:id="rId4"/>
+    <hyperlink ref="M17" r:id="rId5"/>
+    <hyperlink ref="M18" r:id="rId6"/>
+    <hyperlink ref="M20" r:id="rId7"/>
+    <hyperlink ref="M32" r:id="rId8"/>
     <hyperlink ref="M31" r:id="rId9"/>
-    <hyperlink ref="M32" r:id="rId10"/>
-    <hyperlink ref="M33" r:id="rId11"/>
-    <hyperlink ref="M34" r:id="rId12"/>
-    <hyperlink ref="M35" r:id="rId13"/>
-    <hyperlink ref="M36" r:id="rId14"/>
-    <hyperlink ref="M38" r:id="rId15"/>
-    <hyperlink ref="M39" r:id="rId16"/>
-    <hyperlink ref="M41" r:id="rId17"/>
-    <hyperlink ref="M42" r:id="rId18"/>
-    <hyperlink ref="M14" r:id="rId19"/>
+    <hyperlink ref="M33" r:id="rId10"/>
+    <hyperlink ref="M34" r:id="rId11"/>
+    <hyperlink ref="M35" r:id="rId12"/>
+    <hyperlink ref="M30" r:id="rId13"/>
+    <hyperlink ref="M37" r:id="rId14"/>
+    <hyperlink ref="M39" r:id="rId15"/>
+    <hyperlink ref="M40" r:id="rId16"/>
+    <hyperlink ref="M14" r:id="rId17"/>
+    <hyperlink ref="M10" r:id="rId18"/>
+    <hyperlink ref="M11" r:id="rId19"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId20"/>

</xml_diff>

<commit_message>
#16 0R resistor added 10K resistor remove
</commit_message>
<xml_diff>
--- a/Design Files/LTE-Module-v2.0/BOM/Client_BOM_v2.0.xlsx
+++ b/Design Files/LTE-Module-v2.0/BOM/Client_BOM_v2.0.xlsx
@@ -549,13 +549,13 @@
     <t>J4, J5</t>
   </si>
   <si>
-    <t>R1, R2, R12, R15, R16, R19, R20</t>
-  </si>
-  <si>
-    <t>R4</t>
-  </si>
-  <si>
     <t>U3,U4</t>
+  </si>
+  <si>
+    <t>R1, R2, R12</t>
+  </si>
+  <si>
+    <t>R4, R19</t>
   </si>
 </sst>
 </file>
@@ -2710,7 +2710,7 @@
         <v>15</v>
       </c>
       <c r="D30" s="36" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E30" s="37" t="s">
         <v>65</v>
@@ -2731,11 +2731,11 @@
         <v>138</v>
       </c>
       <c r="K30" s="36">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L30" s="36">
         <f>K30*5</f>
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="M30" s="59" t="s">
         <v>148</v>
@@ -2745,7 +2745,7 @@
       </c>
       <c r="O30" s="63">
         <f>N30*L30</f>
-        <v>3.5</v>
+        <v>1.5</v>
       </c>
       <c r="P30" s="36"/>
     </row>
@@ -2807,8 +2807,8 @@
       <c r="C32" s="57" t="s">
         <v>15</v>
       </c>
-      <c r="D32" s="38" t="s">
-        <v>177</v>
+      <c r="D32" s="36" t="s">
+        <v>178</v>
       </c>
       <c r="E32" s="39" t="s">
         <v>60</v>
@@ -2829,11 +2829,11 @@
         <v>133</v>
       </c>
       <c r="K32" s="38">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L32" s="38">
         <f t="shared" ref="L32" si="11">K32*5</f>
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="M32" s="59" t="s">
         <v>148</v>
@@ -2843,7 +2843,7 @@
       </c>
       <c r="O32" s="63">
         <f>N32*L32</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="P32" s="38"/>
     </row>
@@ -3100,7 +3100,7 @@
         <v>17</v>
       </c>
       <c r="D38" s="36" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="E38" s="37" t="s">
         <v>68</v>
@@ -3275,7 +3275,7 @@
       <c r="N42" s="71"/>
       <c r="O42" s="64">
         <f>SUM(O10:O41)</f>
-        <v>47.949999999999996</v>
+        <v>46.449999999999996</v>
       </c>
       <c r="P42" s="41"/>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="N43" s="71"/>
       <c r="O43" s="65">
         <f>O42/5</f>
-        <v>9.59</v>
+        <v>9.2899999999999991</v>
       </c>
       <c r="P43" s="42"/>
     </row>

</xml_diff>

<commit_message>
#16 Antenna change in BOM
</commit_message>
<xml_diff>
--- a/Design Files/LTE-Module-v2.0/BOM/Client_BOM_v2.0.xlsx
+++ b/Design Files/LTE-Module-v2.0/BOM/Client_BOM_v2.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="183">
   <si>
     <t>Component list</t>
   </si>
@@ -483,12 +483,6 @@
     <t>Peripheral</t>
   </si>
   <si>
-    <t xml:space="preserve">SMA Male Antenna </t>
-  </si>
-  <si>
-    <t>Aliexpress</t>
-  </si>
-  <si>
     <t>Custom Supplier</t>
   </si>
   <si>
@@ -556,6 +550,24 @@
   </si>
   <si>
     <t>R4, R19</t>
+  </si>
+  <si>
+    <t>1.8 3dBi Vertical 50W - Antennas ROHS</t>
+  </si>
+  <si>
+    <t>BWGSMJWX105-7KJ</t>
+  </si>
+  <si>
+    <t>BAT WIRELESS</t>
+  </si>
+  <si>
+    <t>2 5dBi 4GAntenna Vertical 2.4GHz 10W - Antennas ROHS</t>
+  </si>
+  <si>
+    <t>801-4G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DreamLNK </t>
   </si>
 </sst>
 </file>
@@ -974,7 +986,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1169,6 +1181,9 @@
     <xf numFmtId="0" fontId="21" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1512,7 +1527,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:P43"/>
+  <dimension ref="A1:P44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="25" customWidth="1"/>
@@ -1523,7 +1538,7 @@
     <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.140625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="18.28515625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="10.5703125" customWidth="1"/>
@@ -1559,7 +1574,7 @@
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="51" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="3"/>
@@ -1581,7 +1596,7 @@
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="52" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="4"/>
@@ -1603,7 +1618,7 @@
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="53" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="G4" s="13"/>
       <c r="H4" s="6"/>
@@ -1747,22 +1762,22 @@
         <v>1</v>
       </c>
       <c r="C10" s="56" t="s">
+        <v>165</v>
+      </c>
+      <c r="D10" s="36" t="s">
+        <v>166</v>
+      </c>
+      <c r="E10" s="36" t="s">
         <v>167</v>
-      </c>
-      <c r="D10" s="36" t="s">
-        <v>168</v>
-      </c>
-      <c r="E10" s="36" t="s">
-        <v>169</v>
       </c>
       <c r="F10" s="36" t="s">
         <v>144</v>
       </c>
       <c r="G10" s="36" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="H10" s="36" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="I10" s="36" t="s">
         <v>143</v>
@@ -1792,7 +1807,7 @@
     <row r="11" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="50">
-        <f t="shared" ref="B11:B41" si="0">ROW(B11) - ROW($B$9)</f>
+        <f t="shared" ref="B11:B42" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="57" t="s">
@@ -1802,13 +1817,13 @@
         <v>19</v>
       </c>
       <c r="E11" s="38" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="F11" s="38" t="s">
         <v>71</v>
       </c>
       <c r="G11" s="38" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="H11" s="38" t="s">
         <v>113</v>
@@ -1817,7 +1832,7 @@
         <v>143</v>
       </c>
       <c r="J11" s="38" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="K11" s="38">
         <v>1</v>
@@ -1897,7 +1912,7 @@
         <v>7</v>
       </c>
       <c r="D13" s="38" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="E13" s="39" t="s">
         <v>45</v>
@@ -1949,16 +1964,16 @@
         <v>21</v>
       </c>
       <c r="E14" s="36" t="s">
+        <v>158</v>
+      </c>
+      <c r="F14" s="36" t="s">
+        <v>159</v>
+      </c>
+      <c r="G14" s="36" t="s">
         <v>160</v>
       </c>
-      <c r="F14" s="36" t="s">
+      <c r="H14" s="36" t="s">
         <v>161</v>
-      </c>
-      <c r="G14" s="36" t="s">
-        <v>162</v>
-      </c>
-      <c r="H14" s="36" t="s">
-        <v>163</v>
       </c>
       <c r="I14" s="36" t="s">
         <v>143</v>
@@ -2219,7 +2234,7 @@
         <v>10</v>
       </c>
       <c r="M19" s="60" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="N19" s="62"/>
       <c r="O19" s="61">
@@ -2315,7 +2330,7 @@
         <v>5</v>
       </c>
       <c r="M21" s="60" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="N21" s="62"/>
       <c r="O21" s="61">
@@ -2362,7 +2377,7 @@
         <v>5</v>
       </c>
       <c r="M22" s="60" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="N22" s="61"/>
       <c r="O22" s="61">
@@ -2384,16 +2399,16 @@
         <v>30</v>
       </c>
       <c r="E23" s="38" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="F23" s="38" t="s">
         <v>144</v>
       </c>
       <c r="G23" s="38" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="H23" s="38" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="I23" s="36" t="s">
         <v>143</v>
@@ -2409,7 +2424,7 @@
         <v>5</v>
       </c>
       <c r="M23" s="60" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="N23" s="62"/>
       <c r="O23" s="61">
@@ -2522,7 +2537,7 @@
         <v>12</v>
       </c>
       <c r="D26" s="36" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E26" s="37" t="s">
         <v>56</v>
@@ -2550,7 +2565,7 @@
         <v>10</v>
       </c>
       <c r="M26" s="60" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="N26" s="61"/>
       <c r="O26" s="61">
@@ -2597,7 +2612,7 @@
         <v>5</v>
       </c>
       <c r="M27" s="60" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="N27" s="61"/>
       <c r="O27" s="61">
@@ -2644,7 +2659,7 @@
         <v>5</v>
       </c>
       <c r="M28" s="60" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="N28" s="62"/>
       <c r="O28" s="61">
@@ -2691,7 +2706,7 @@
         <v>20</v>
       </c>
       <c r="M29" s="60" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="N29" s="61"/>
       <c r="O29" s="61">
@@ -2710,7 +2725,7 @@
         <v>15</v>
       </c>
       <c r="D30" s="36" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="E30" s="37" t="s">
         <v>65</v>
@@ -2808,7 +2823,7 @@
         <v>15</v>
       </c>
       <c r="D32" s="36" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="E32" s="39" t="s">
         <v>60</v>
@@ -2891,7 +2906,7 @@
         <v>0.1</v>
       </c>
       <c r="O33" s="63">
-        <f t="shared" ref="O33:O40" si="13">N33*L33</f>
+        <f t="shared" ref="O33:O39" si="13">N33*L33</f>
         <v>1</v>
       </c>
       <c r="P33" s="38"/>
@@ -3032,7 +3047,7 @@
         <v>5</v>
       </c>
       <c r="M36" s="60" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="N36" s="62"/>
       <c r="O36" s="63">
@@ -3100,7 +3115,7 @@
         <v>17</v>
       </c>
       <c r="D38" s="36" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="E38" s="37" t="s">
         <v>68</v>
@@ -3128,7 +3143,7 @@
         <v>5</v>
       </c>
       <c r="M38" s="60" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="N38" s="61"/>
       <c r="O38" s="63">
@@ -3171,7 +3186,7 @@
         <v>1</v>
       </c>
       <c r="L39" s="38">
-        <f t="shared" ref="L39:L40" si="16">K39*5</f>
+        <f t="shared" ref="L39:L41" si="16">K39*5</f>
         <v>5</v>
       </c>
       <c r="M39" s="59" t="s">
@@ -3186,7 +3201,7 @@
       </c>
       <c r="P39" s="38"/>
     </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
       <c r="B40" s="66">
         <f t="shared" si="0"/>
@@ -3198,20 +3213,22 @@
       <c r="D40" s="38" t="s">
         <v>143</v>
       </c>
-      <c r="E40" s="38" t="s">
-        <v>143</v>
-      </c>
-      <c r="F40" s="38" t="s">
-        <v>143</v>
-      </c>
-      <c r="G40" s="38" t="s">
-        <v>154</v>
-      </c>
-      <c r="H40" s="38"/>
+      <c r="E40" s="72" t="s">
+        <v>177</v>
+      </c>
+      <c r="F40" s="72"/>
+      <c r="G40" s="72" t="s">
+        <v>178</v>
+      </c>
+      <c r="H40" s="72" t="s">
+        <v>179</v>
+      </c>
       <c r="I40" s="36" t="s">
         <v>143</v>
       </c>
-      <c r="J40" s="38"/>
+      <c r="J40" s="38" t="s">
+        <v>143</v>
+      </c>
       <c r="K40" s="38">
         <v>1</v>
       </c>
@@ -3219,19 +3236,17 @@
         <f t="shared" si="16"/>
         <v>5</v>
       </c>
-      <c r="M40" s="59" t="s">
-        <v>155</v>
-      </c>
-      <c r="N40" s="62">
-        <v>0.8</v>
-      </c>
+      <c r="M40" s="60" t="s">
+        <v>154</v>
+      </c>
+      <c r="N40" s="61"/>
       <c r="O40" s="63">
-        <f t="shared" si="13"/>
-        <v>4</v>
+        <f t="shared" ref="O40:O41" si="17">N40*L40</f>
+        <v>0</v>
       </c>
       <c r="P40" s="38"/>
     </row>
-    <row r="41" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="66">
         <f t="shared" si="0"/>
@@ -3240,74 +3255,121 @@
       <c r="C41" s="57" t="s">
         <v>153</v>
       </c>
-      <c r="D41" s="38"/>
-      <c r="E41" s="38"/>
-      <c r="F41" s="38"/>
-      <c r="G41" s="38"/>
-      <c r="H41" s="38"/>
+      <c r="D41" s="38" t="s">
+        <v>143</v>
+      </c>
+      <c r="E41" s="38" t="s">
+        <v>180</v>
+      </c>
+      <c r="F41" s="38" t="s">
+        <v>143</v>
+      </c>
+      <c r="G41" s="38" t="s">
+        <v>181</v>
+      </c>
+      <c r="H41" s="38" t="s">
+        <v>182</v>
+      </c>
       <c r="I41" s="36" t="s">
         <v>143</v>
       </c>
-      <c r="J41" s="38"/>
-      <c r="K41" s="38"/>
-      <c r="L41" s="38"/>
-      <c r="M41" s="59"/>
-      <c r="N41" s="62"/>
-      <c r="O41" s="63"/>
+      <c r="J41" s="38" t="s">
+        <v>143</v>
+      </c>
+      <c r="K41" s="38">
+        <v>1</v>
+      </c>
+      <c r="L41" s="38">
+        <f t="shared" si="16"/>
+        <v>5</v>
+      </c>
+      <c r="M41" s="60" t="s">
+        <v>154</v>
+      </c>
+      <c r="N41" s="61"/>
+      <c r="O41" s="63">
+        <f t="shared" ref="O41" si="18">N41*L41</f>
+        <v>0</v>
+      </c>
       <c r="P41" s="38"/>
     </row>
-    <row r="42" spans="1:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
-      <c r="B42" s="31"/>
-      <c r="C42" s="48"/>
-      <c r="D42" s="32"/>
-      <c r="E42" s="33"/>
-      <c r="F42" s="34"/>
-      <c r="G42" s="35"/>
-      <c r="H42" s="34"/>
-      <c r="I42" s="35"/>
-      <c r="J42" s="35"/>
-      <c r="K42" s="35"/>
-      <c r="L42" s="70" t="s">
-        <v>151</v>
-      </c>
-      <c r="M42" s="71"/>
-      <c r="N42" s="71"/>
-      <c r="O42" s="64">
-        <f>SUM(O10:O41)</f>
-        <v>46.449999999999996</v>
-      </c>
-      <c r="P42" s="41"/>
+      <c r="B42" s="66">
+        <f t="shared" si="0"/>
+        <v>33</v>
+      </c>
+      <c r="C42" s="57" t="s">
+        <v>153</v>
+      </c>
+      <c r="D42" s="38"/>
+      <c r="E42" s="38"/>
+      <c r="F42" s="38"/>
+      <c r="G42" s="38"/>
+      <c r="H42" s="38"/>
+      <c r="I42" s="36" t="s">
+        <v>143</v>
+      </c>
+      <c r="J42" s="38"/>
+      <c r="K42" s="38"/>
+      <c r="L42" s="38"/>
+      <c r="M42" s="59"/>
+      <c r="N42" s="62"/>
+      <c r="O42" s="63"/>
+      <c r="P42" s="38"/>
     </row>
     <row r="43" spans="1:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
-      <c r="B43" s="24"/>
-      <c r="C43" s="49"/>
-      <c r="D43" s="8"/>
-      <c r="E43" s="9"/>
-      <c r="F43" s="9"/>
-      <c r="G43" s="9"/>
-      <c r="H43" s="9"/>
-      <c r="I43" s="9"/>
-      <c r="J43" s="9"/>
-      <c r="K43" s="9"/>
+      <c r="B43" s="31"/>
+      <c r="C43" s="48"/>
+      <c r="D43" s="32"/>
+      <c r="E43" s="33"/>
+      <c r="F43" s="34"/>
+      <c r="G43" s="35"/>
+      <c r="H43" s="34"/>
+      <c r="I43" s="35"/>
+      <c r="J43" s="35"/>
+      <c r="K43" s="35"/>
       <c r="L43" s="70" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="M43" s="71"/>
       <c r="N43" s="71"/>
-      <c r="O43" s="65">
-        <f>O42/5</f>
-        <v>9.2899999999999991</v>
-      </c>
-      <c r="P43" s="42"/>
+      <c r="O43" s="64">
+        <f>SUM(O10:O42)</f>
+        <v>42.449999999999996</v>
+      </c>
+      <c r="P43" s="41"/>
+    </row>
+    <row r="44" spans="1:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="1"/>
+      <c r="B44" s="24"/>
+      <c r="C44" s="49"/>
+      <c r="D44" s="8"/>
+      <c r="E44" s="9"/>
+      <c r="F44" s="9"/>
+      <c r="G44" s="9"/>
+      <c r="H44" s="9"/>
+      <c r="I44" s="9"/>
+      <c r="J44" s="9"/>
+      <c r="K44" s="9"/>
+      <c r="L44" s="70" t="s">
+        <v>152</v>
+      </c>
+      <c r="M44" s="71"/>
+      <c r="N44" s="71"/>
+      <c r="O44" s="65">
+        <f>O43/5</f>
+        <v>8.4899999999999984</v>
+      </c>
+      <c r="P44" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="J1:P1"/>
     <mergeCell ref="P3:P8"/>
-    <mergeCell ref="L42:N42"/>
     <mergeCell ref="L43:N43"/>
+    <mergeCell ref="L44:N44"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="M12" r:id="rId1"/>
@@ -3325,13 +3387,12 @@
     <hyperlink ref="M30" r:id="rId13"/>
     <hyperlink ref="M37" r:id="rId14"/>
     <hyperlink ref="M39" r:id="rId15"/>
-    <hyperlink ref="M40" r:id="rId16"/>
-    <hyperlink ref="M14" r:id="rId17"/>
-    <hyperlink ref="M10" r:id="rId18"/>
-    <hyperlink ref="M11" r:id="rId19"/>
+    <hyperlink ref="M14" r:id="rId16"/>
+    <hyperlink ref="M10" r:id="rId17"/>
+    <hyperlink ref="M11" r:id="rId18"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId20"/>
-  <drawing r:id="rId21"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId19"/>
+  <drawing r:id="rId20"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
#16 Client BOM Updated.
</commit_message>
<xml_diff>
--- a/Design Files/LTE-Module-v2.0/BOM/Client_BOM_v2.0.xlsx
+++ b/Design Files/LTE-Module-v2.0/BOM/Client_BOM_v2.0.xlsx
@@ -51,9 +51,6 @@
     <t>Fuse</t>
   </si>
   <si>
-    <t>Connector</t>
-  </si>
-  <si>
     <t>Pogo Connector</t>
   </si>
   <si>
@@ -486,12 +483,6 @@
     <t>Custom Supplier</t>
   </si>
   <si>
-    <t>1 Inner bore SMA Board Edge Bend -55℃~+155℃ 50Ω Plugin RF Connectors / Coaxial Connectors ROHS</t>
-  </si>
-  <si>
-    <t>HJ-SMA508</t>
-  </si>
-  <si>
     <t>HJ Tech</t>
   </si>
   <si>
@@ -568,6 +559,15 @@
   </si>
   <si>
     <t xml:space="preserve">DreamLNK </t>
+  </si>
+  <si>
+    <t>SMA Connector</t>
+  </si>
+  <si>
+    <t>1 Inner bore SMA Board Edge Bend 11mm 5.35mm Plugin RF Connectors / Coaxial Connectors ROHS</t>
+  </si>
+  <si>
+    <t>HJ-SMA175</t>
   </si>
 </sst>
 </file>
@@ -1165,6 +1165,9 @@
     <xf numFmtId="0" fontId="10" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1181,9 +1184,6 @@
     <xf numFmtId="0" fontId="21" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1557,13 +1557,13 @@
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="67"/>
-      <c r="P1" s="67"/>
+      <c r="J1" s="68"/>
+      <c r="K1" s="68"/>
+      <c r="L1" s="68"/>
+      <c r="M1" s="68"/>
+      <c r="N1" s="68"/>
+      <c r="O1" s="68"/>
+      <c r="P1" s="68"/>
     </row>
     <row r="2" spans="1:16" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="51" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="3"/>
@@ -1596,7 +1596,7 @@
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="52" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="4"/>
@@ -1607,7 +1607,7 @@
       <c r="M3" s="4"/>
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
-      <c r="P3" s="68"/>
+      <c r="P3" s="69"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1618,7 +1618,7 @@
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="53" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="G4" s="13"/>
       <c r="H4" s="6"/>
@@ -1629,7 +1629,7 @@
       <c r="M4" s="58"/>
       <c r="N4" s="58"/>
       <c r="O4" s="58"/>
-      <c r="P4" s="69"/>
+      <c r="P4" s="70"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1651,7 +1651,7 @@
       <c r="M5" s="58"/>
       <c r="N5" s="58"/>
       <c r="O5" s="58"/>
-      <c r="P5" s="69"/>
+      <c r="P5" s="70"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -1669,7 +1669,7 @@
       <c r="M6" s="58"/>
       <c r="N6" s="58"/>
       <c r="O6" s="58"/>
-      <c r="P6" s="69"/>
+      <c r="P6" s="70"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -1687,7 +1687,7 @@
       <c r="M7" s="7"/>
       <c r="N7" s="7"/>
       <c r="O7" s="7"/>
-      <c r="P7" s="69"/>
+      <c r="P7" s="70"/>
     </row>
     <row r="8" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1705,7 +1705,7 @@
       <c r="M8" s="7"/>
       <c r="N8" s="7"/>
       <c r="O8" s="7"/>
-      <c r="P8" s="69"/>
+      <c r="P8" s="70"/>
     </row>
     <row r="9" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -1716,43 +1716,43 @@
         <v>6</v>
       </c>
       <c r="D9" s="29" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E9" s="30" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F9" s="29" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G9" s="30" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H9" s="29" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I9" s="29" t="s">
+        <v>139</v>
+      </c>
+      <c r="J9" s="29" t="s">
+        <v>141</v>
+      </c>
+      <c r="K9" s="29" t="s">
+        <v>138</v>
+      </c>
+      <c r="L9" s="29" t="s">
         <v>140</v>
       </c>
-      <c r="J9" s="29" t="s">
-        <v>142</v>
-      </c>
-      <c r="K9" s="29" t="s">
-        <v>139</v>
-      </c>
-      <c r="L9" s="29" t="s">
-        <v>141</v>
-      </c>
       <c r="M9" s="29" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="N9" s="29" t="s">
+        <v>148</v>
+      </c>
+      <c r="O9" s="29" t="s">
         <v>149</v>
       </c>
-      <c r="O9" s="29" t="s">
-        <v>150</v>
-      </c>
       <c r="P9" s="29" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1762,28 +1762,28 @@
         <v>1</v>
       </c>
       <c r="C10" s="56" t="s">
+        <v>162</v>
+      </c>
+      <c r="D10" s="36" t="s">
+        <v>163</v>
+      </c>
+      <c r="E10" s="36" t="s">
+        <v>164</v>
+      </c>
+      <c r="F10" s="36" t="s">
+        <v>143</v>
+      </c>
+      <c r="G10" s="36" t="s">
         <v>165</v>
       </c>
-      <c r="D10" s="36" t="s">
+      <c r="H10" s="36" t="s">
         <v>166</v>
       </c>
-      <c r="E10" s="36" t="s">
-        <v>167</v>
-      </c>
-      <c r="F10" s="36" t="s">
-        <v>144</v>
-      </c>
-      <c r="G10" s="36" t="s">
-        <v>168</v>
-      </c>
-      <c r="H10" s="36" t="s">
-        <v>169</v>
-      </c>
       <c r="I10" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J10" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="K10" s="36">
         <v>1</v>
@@ -1793,7 +1793,7 @@
         <v>5</v>
       </c>
       <c r="M10" s="59" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="N10" s="61">
         <v>1.59</v>
@@ -1814,25 +1814,25 @@
         <v>7</v>
       </c>
       <c r="D11" s="38" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E11" s="38" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="F11" s="38" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G11" s="38" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="H11" s="38" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I11" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J11" s="38" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="K11" s="38">
         <v>1</v>
@@ -1842,7 +1842,7 @@
         <v>5</v>
       </c>
       <c r="M11" s="60" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="N11" s="62">
         <v>0.1</v>
@@ -1863,25 +1863,25 @@
         <v>7</v>
       </c>
       <c r="D12" s="36" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E12" s="37" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F12" s="36" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G12" s="37" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H12" s="36" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I12" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J12" s="36" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="K12" s="36">
         <v>1</v>
@@ -1891,7 +1891,7 @@
         <v>5</v>
       </c>
       <c r="M12" s="59" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="N12" s="61">
         <v>0.1</v>
@@ -1912,25 +1912,25 @@
         <v>7</v>
       </c>
       <c r="D13" s="38" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E13" s="39" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F13" s="38" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G13" s="39" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H13" s="38" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I13" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J13" s="38" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="K13" s="38">
         <v>6</v>
@@ -1940,7 +1940,7 @@
         <v>30</v>
       </c>
       <c r="M13" s="60" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="N13" s="62">
         <v>0.1</v>
@@ -1961,25 +1961,25 @@
         <v>7</v>
       </c>
       <c r="D14" s="36" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E14" s="36" t="s">
+        <v>155</v>
+      </c>
+      <c r="F14" s="36" t="s">
+        <v>156</v>
+      </c>
+      <c r="G14" s="36" t="s">
+        <v>157</v>
+      </c>
+      <c r="H14" s="36" t="s">
         <v>158</v>
       </c>
-      <c r="F14" s="36" t="s">
-        <v>159</v>
-      </c>
-      <c r="G14" s="36" t="s">
-        <v>160</v>
-      </c>
-      <c r="H14" s="36" t="s">
-        <v>161</v>
-      </c>
       <c r="I14" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J14" s="36" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K14" s="36">
         <v>1</v>
@@ -1989,7 +1989,7 @@
         <v>5</v>
       </c>
       <c r="M14" s="60" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="N14" s="61">
         <v>1.04</v>
@@ -2010,25 +2010,25 @@
         <v>7</v>
       </c>
       <c r="D15" s="38" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E15" s="39" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F15" s="38" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G15" s="39" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H15" s="38" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I15" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J15" s="38" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="K15" s="38">
         <v>1</v>
@@ -2038,7 +2038,7 @@
         <v>5</v>
       </c>
       <c r="M15" s="60" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="N15" s="62">
         <v>0.1</v>
@@ -2059,25 +2059,25 @@
         <v>7</v>
       </c>
       <c r="D16" s="36" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E16" s="37" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F16" s="36" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G16" s="37" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H16" s="36" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I16" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J16" s="36" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="K16" s="36">
         <v>3</v>
@@ -2087,7 +2087,7 @@
         <v>15</v>
       </c>
       <c r="M16" s="59" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="N16" s="61">
         <v>0.1</v>
@@ -2108,25 +2108,25 @@
         <v>7</v>
       </c>
       <c r="D17" s="38" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E17" s="39" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F17" s="38" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G17" s="39" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H17" s="38" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="I17" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J17" s="38" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K17" s="38">
         <v>2</v>
@@ -2136,7 +2136,7 @@
         <v>10</v>
       </c>
       <c r="M17" s="59" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="N17" s="62">
         <v>0.11</v>
@@ -2157,25 +2157,25 @@
         <v>8</v>
       </c>
       <c r="D18" s="36" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E18" s="37" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F18" s="36" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G18" s="37" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H18" s="36" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I18" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J18" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="K18" s="36">
         <v>1</v>
@@ -2185,7 +2185,7 @@
         <v>5</v>
       </c>
       <c r="M18" s="59" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="N18" s="61">
         <v>0.23</v>
@@ -2206,25 +2206,25 @@
         <v>8</v>
       </c>
       <c r="D19" s="38" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E19" s="39" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F19" s="38" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G19" s="39" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H19" s="38" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="I19" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J19" s="38" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="K19" s="38">
         <v>2</v>
@@ -2234,7 +2234,7 @@
         <v>10</v>
       </c>
       <c r="M19" s="60" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="N19" s="62"/>
       <c r="O19" s="61">
@@ -2253,25 +2253,25 @@
         <v>8</v>
       </c>
       <c r="D20" s="36" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E20" s="37" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F20" s="36" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G20" s="37" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H20" s="36" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="I20" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J20" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="K20" s="36">
         <v>1</v>
@@ -2281,7 +2281,7 @@
         <v>5</v>
       </c>
       <c r="M20" s="59" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="N20" s="61">
         <v>0.48</v>
@@ -2302,25 +2302,25 @@
         <v>8</v>
       </c>
       <c r="D21" s="38" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E21" s="39" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F21" s="38" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G21" s="39" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H21" s="38" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I21" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J21" s="38" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="K21" s="38">
         <v>1</v>
@@ -2330,7 +2330,7 @@
         <v>5</v>
       </c>
       <c r="M21" s="60" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="N21" s="62"/>
       <c r="O21" s="61">
@@ -2349,25 +2349,25 @@
         <v>9</v>
       </c>
       <c r="D22" s="36" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E22" s="37" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F22" s="36" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G22" s="37" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="H22" s="36" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I22" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J22" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="K22" s="36">
         <v>1</v>
@@ -2377,7 +2377,7 @@
         <v>5</v>
       </c>
       <c r="M22" s="60" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="N22" s="61"/>
       <c r="O22" s="61">
@@ -2386,35 +2386,35 @@
       </c>
       <c r="P22" s="36"/>
     </row>
-    <row r="23" spans="1:16" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:16" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="50">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="C23" s="57" t="s">
-        <v>10</v>
+        <v>180</v>
       </c>
       <c r="D23" s="38" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E23" s="38" t="s">
-        <v>155</v>
+        <v>181</v>
       </c>
       <c r="F23" s="38" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G23" s="38" t="s">
-        <v>156</v>
+        <v>182</v>
       </c>
       <c r="H23" s="38" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="I23" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J23" s="38" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="K23" s="38">
         <v>1</v>
@@ -2424,7 +2424,7 @@
         <v>5</v>
       </c>
       <c r="M23" s="60" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="N23" s="62"/>
       <c r="O23" s="61">
@@ -2440,28 +2440,28 @@
         <v>15</v>
       </c>
       <c r="C24" s="56" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D24" s="36" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E24" s="37" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F24" s="55" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G24" s="37" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="H24" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="I24" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J24" s="55" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="K24" s="36">
         <v>1</v>
@@ -2471,7 +2471,7 @@
         <v>5</v>
       </c>
       <c r="M24" s="55" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="N24" s="61"/>
       <c r="O24" s="61">
@@ -2487,28 +2487,28 @@
         <v>16</v>
       </c>
       <c r="C25" s="57" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D25" s="38" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E25" s="39" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F25" s="38" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G25" s="39" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H25" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="I25" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J25" s="55" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="K25" s="38">
         <v>1</v>
@@ -2518,7 +2518,7 @@
         <v>5</v>
       </c>
       <c r="M25" s="55" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="N25" s="62"/>
       <c r="O25" s="61">
@@ -2534,28 +2534,28 @@
         <v>17</v>
       </c>
       <c r="C26" s="56" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D26" s="36" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="E26" s="37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F26" s="36" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G26" s="37" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H26" s="36" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="I26" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J26" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="K26" s="36">
         <v>2</v>
@@ -2565,7 +2565,7 @@
         <v>10</v>
       </c>
       <c r="M26" s="60" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="N26" s="61"/>
       <c r="O26" s="61">
@@ -2581,28 +2581,28 @@
         <v>18</v>
       </c>
       <c r="C27" s="56" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D27" s="36" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E27" s="37" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F27" s="36" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G27" s="37" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="H27" s="36" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I27" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J27" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="K27" s="36">
         <v>1</v>
@@ -2612,7 +2612,7 @@
         <v>5</v>
       </c>
       <c r="M27" s="60" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="N27" s="61"/>
       <c r="O27" s="61">
@@ -2628,28 +2628,28 @@
         <v>19</v>
       </c>
       <c r="C28" s="57" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D28" s="38" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E28" s="39" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F28" s="38" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G28" s="39" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H28" s="38" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I28" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J28" s="38" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="K28" s="38">
         <v>1</v>
@@ -2659,7 +2659,7 @@
         <v>5</v>
       </c>
       <c r="M28" s="60" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="N28" s="62"/>
       <c r="O28" s="61">
@@ -2675,28 +2675,28 @@
         <v>20</v>
       </c>
       <c r="C29" s="56" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D29" s="36" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E29" s="37" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F29" s="36" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G29" s="37" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H29" s="36" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="I29" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J29" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="K29" s="36">
         <v>4</v>
@@ -2706,7 +2706,7 @@
         <v>20</v>
       </c>
       <c r="M29" s="60" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="N29" s="61"/>
       <c r="O29" s="61">
@@ -2722,28 +2722,28 @@
         <v>21</v>
       </c>
       <c r="C30" s="56" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D30" s="36" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="E30" s="37" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F30" s="36" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G30" s="37" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H30" s="36" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I30" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J30" s="36" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K30" s="36">
         <v>3</v>
@@ -2753,7 +2753,7 @@
         <v>15</v>
       </c>
       <c r="M30" s="59" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="N30" s="62">
         <v>0.1</v>
@@ -2771,28 +2771,28 @@
         <v>22</v>
       </c>
       <c r="C31" s="56" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D31" s="36" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E31" s="37" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F31" s="36" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G31" s="37" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H31" s="36" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I31" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J31" s="36" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="K31" s="36">
         <v>2</v>
@@ -2802,7 +2802,7 @@
         <v>10</v>
       </c>
       <c r="M31" s="59" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="N31" s="62">
         <v>0.1</v>
@@ -2820,28 +2820,28 @@
         <v>23</v>
       </c>
       <c r="C32" s="57" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D32" s="36" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="E32" s="39" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F32" s="38" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G32" s="39" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H32" s="38" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I32" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J32" s="38" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K32" s="38">
         <v>2</v>
@@ -2851,7 +2851,7 @@
         <v>10</v>
       </c>
       <c r="M32" s="59" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="N32" s="62">
         <v>0.1</v>
@@ -2869,28 +2869,28 @@
         <v>24</v>
       </c>
       <c r="C33" s="57" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D33" s="38" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E33" s="39" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F33" s="38" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G33" s="39" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H33" s="38" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I33" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J33" s="38" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="K33" s="38">
         <v>2</v>
@@ -2900,7 +2900,7 @@
         <v>10</v>
       </c>
       <c r="M33" s="59" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="N33" s="62">
         <v>0.1</v>
@@ -2918,28 +2918,28 @@
         <v>25</v>
       </c>
       <c r="C34" s="56" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D34" s="36" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E34" s="37" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F34" s="36" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G34" s="37" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H34" s="36" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I34" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J34" s="36" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="K34" s="36">
         <v>4</v>
@@ -2949,7 +2949,7 @@
         <v>20</v>
       </c>
       <c r="M34" s="59" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="N34" s="62">
         <v>0.1</v>
@@ -2967,28 +2967,28 @@
         <v>26</v>
       </c>
       <c r="C35" s="56" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D35" s="38" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E35" s="39" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F35" s="38" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G35" s="39" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H35" s="38" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I35" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J35" s="38" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="K35" s="38">
         <v>4</v>
@@ -2998,7 +2998,7 @@
         <v>20</v>
       </c>
       <c r="M35" s="59" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="N35" s="62">
         <v>0.1</v>
@@ -3016,28 +3016,28 @@
         <v>27</v>
       </c>
       <c r="C36" s="57" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D36" s="38" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E36" s="39" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F36" s="38" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G36" s="39" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H36" s="38" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I36" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J36" s="38" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="K36" s="38">
         <v>1</v>
@@ -3047,7 +3047,7 @@
         <v>5</v>
       </c>
       <c r="M36" s="60" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="N36" s="62"/>
       <c r="O36" s="63">
@@ -3063,28 +3063,28 @@
         <v>28</v>
       </c>
       <c r="C37" s="56" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D37" s="36" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E37" s="37" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F37" s="36" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G37" s="37" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H37" s="36" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I37" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J37" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="K37" s="36">
         <v>1</v>
@@ -3094,7 +3094,7 @@
         <v>5</v>
       </c>
       <c r="M37" s="59" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="N37" s="61">
         <v>0.95</v>
@@ -3112,28 +3112,28 @@
         <v>29</v>
       </c>
       <c r="C38" s="56" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D38" s="36" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="E38" s="37" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F38" s="36" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G38" s="37" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H38" s="36" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I38" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J38" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="K38" s="36">
         <v>1</v>
@@ -3143,7 +3143,7 @@
         <v>5</v>
       </c>
       <c r="M38" s="60" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="N38" s="61"/>
       <c r="O38" s="63">
@@ -3159,28 +3159,28 @@
         <v>30</v>
       </c>
       <c r="C39" s="57" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D39" s="38" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E39" s="39" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F39" s="38" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G39" s="39" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H39" s="38" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I39" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J39" s="38" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="K39" s="38">
         <v>1</v>
@@ -3190,7 +3190,7 @@
         <v>5</v>
       </c>
       <c r="M39" s="59" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="N39" s="62">
         <v>1.08</v>
@@ -3208,26 +3208,26 @@
         <v>31</v>
       </c>
       <c r="C40" s="57" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D40" s="38" t="s">
-        <v>143</v>
-      </c>
-      <c r="E40" s="72" t="s">
-        <v>177</v>
-      </c>
-      <c r="F40" s="72"/>
-      <c r="G40" s="72" t="s">
-        <v>178</v>
-      </c>
-      <c r="H40" s="72" t="s">
-        <v>179</v>
+        <v>142</v>
+      </c>
+      <c r="E40" s="67" t="s">
+        <v>174</v>
+      </c>
+      <c r="F40" s="67"/>
+      <c r="G40" s="67" t="s">
+        <v>175</v>
+      </c>
+      <c r="H40" s="67" t="s">
+        <v>176</v>
       </c>
       <c r="I40" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J40" s="38" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="K40" s="38">
         <v>1</v>
@@ -3237,11 +3237,11 @@
         <v>5</v>
       </c>
       <c r="M40" s="60" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="N40" s="61"/>
       <c r="O40" s="63">
-        <f t="shared" ref="O40:O41" si="17">N40*L40</f>
+        <f t="shared" ref="O40" si="17">N40*L40</f>
         <v>0</v>
       </c>
       <c r="P40" s="38"/>
@@ -3253,28 +3253,28 @@
         <v>32</v>
       </c>
       <c r="C41" s="57" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D41" s="38" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E41" s="38" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="F41" s="38" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G41" s="38" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="H41" s="38" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="I41" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J41" s="38" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="K41" s="38">
         <v>1</v>
@@ -3284,7 +3284,7 @@
         <v>5</v>
       </c>
       <c r="M41" s="60" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="N41" s="61"/>
       <c r="O41" s="63">
@@ -3300,7 +3300,7 @@
         <v>33</v>
       </c>
       <c r="C42" s="57" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D42" s="38"/>
       <c r="E42" s="38"/>
@@ -3308,7 +3308,7 @@
       <c r="G42" s="38"/>
       <c r="H42" s="38"/>
       <c r="I42" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J42" s="38"/>
       <c r="K42" s="38"/>
@@ -3330,11 +3330,11 @@
       <c r="I43" s="35"/>
       <c r="J43" s="35"/>
       <c r="K43" s="35"/>
-      <c r="L43" s="70" t="s">
-        <v>151</v>
-      </c>
-      <c r="M43" s="71"/>
-      <c r="N43" s="71"/>
+      <c r="L43" s="71" t="s">
+        <v>150</v>
+      </c>
+      <c r="M43" s="72"/>
+      <c r="N43" s="72"/>
       <c r="O43" s="64">
         <f>SUM(O10:O42)</f>
         <v>42.449999999999996</v>
@@ -3353,11 +3353,11 @@
       <c r="I44" s="9"/>
       <c r="J44" s="9"/>
       <c r="K44" s="9"/>
-      <c r="L44" s="70" t="s">
-        <v>152</v>
-      </c>
-      <c r="M44" s="71"/>
-      <c r="N44" s="71"/>
+      <c r="L44" s="71" t="s">
+        <v>151</v>
+      </c>
+      <c r="M44" s="72"/>
+      <c r="N44" s="72"/>
       <c r="O44" s="65">
         <f>O43/5</f>
         <v>8.4899999999999984</v>

</xml_diff>

<commit_message>
#31 Client BOM Updated
</commit_message>
<xml_diff>
--- a/Design Files/LTE-Module-v2.0/BOM/Client_BOM_v2.0.xlsx
+++ b/Design Files/LTE-Module-v2.0/BOM/Client_BOM_v2.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="183">
   <si>
     <t>Component list</t>
   </si>
@@ -1527,7 +1527,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:P44"/>
+  <dimension ref="A1:P43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="25" customWidth="1"/>
@@ -1807,7 +1807,7 @@
     <row r="11" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="50">
-        <f t="shared" ref="B11:B42" si="0">ROW(B11) - ROW($B$9)</f>
+        <f t="shared" ref="B11:B41" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="57" t="s">
@@ -3246,7 +3246,7 @@
       </c>
       <c r="P40" s="38"/>
     </row>
-    <row r="41" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
       <c r="B41" s="66">
         <f t="shared" si="0"/>
@@ -3293,83 +3293,58 @@
       </c>
       <c r="P41" s="38"/>
     </row>
-    <row r="42" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
-      <c r="B42" s="66">
-        <f t="shared" si="0"/>
-        <v>33</v>
-      </c>
-      <c r="C42" s="57" t="s">
-        <v>152</v>
-      </c>
-      <c r="D42" s="38"/>
-      <c r="E42" s="38"/>
-      <c r="F42" s="38"/>
-      <c r="G42" s="38"/>
-      <c r="H42" s="38"/>
-      <c r="I42" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J42" s="38"/>
-      <c r="K42" s="38"/>
-      <c r="L42" s="38"/>
-      <c r="M42" s="59"/>
-      <c r="N42" s="62"/>
-      <c r="O42" s="63"/>
-      <c r="P42" s="38"/>
+      <c r="B42" s="31"/>
+      <c r="C42" s="48"/>
+      <c r="D42" s="32"/>
+      <c r="E42" s="33"/>
+      <c r="F42" s="34"/>
+      <c r="G42" s="35"/>
+      <c r="H42" s="34"/>
+      <c r="I42" s="35"/>
+      <c r="J42" s="35"/>
+      <c r="K42" s="35"/>
+      <c r="L42" s="71" t="s">
+        <v>150</v>
+      </c>
+      <c r="M42" s="72"/>
+      <c r="N42" s="72"/>
+      <c r="O42" s="64">
+        <f>SUM(O10:O41)</f>
+        <v>42.449999999999996</v>
+      </c>
+      <c r="P42" s="41"/>
     </row>
     <row r="43" spans="1:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
-      <c r="B43" s="31"/>
-      <c r="C43" s="48"/>
-      <c r="D43" s="32"/>
-      <c r="E43" s="33"/>
-      <c r="F43" s="34"/>
-      <c r="G43" s="35"/>
-      <c r="H43" s="34"/>
-      <c r="I43" s="35"/>
-      <c r="J43" s="35"/>
-      <c r="K43" s="35"/>
+      <c r="B43" s="24"/>
+      <c r="C43" s="49"/>
+      <c r="D43" s="8"/>
+      <c r="E43" s="9"/>
+      <c r="F43" s="9"/>
+      <c r="G43" s="9"/>
+      <c r="H43" s="9"/>
+      <c r="I43" s="9"/>
+      <c r="J43" s="9"/>
+      <c r="K43" s="9"/>
       <c r="L43" s="71" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="M43" s="72"/>
       <c r="N43" s="72"/>
-      <c r="O43" s="64">
-        <f>SUM(O10:O42)</f>
-        <v>42.449999999999996</v>
-      </c>
-      <c r="P43" s="41"/>
-    </row>
-    <row r="44" spans="1:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="1"/>
-      <c r="B44" s="24"/>
-      <c r="C44" s="49"/>
-      <c r="D44" s="8"/>
-      <c r="E44" s="9"/>
-      <c r="F44" s="9"/>
-      <c r="G44" s="9"/>
-      <c r="H44" s="9"/>
-      <c r="I44" s="9"/>
-      <c r="J44" s="9"/>
-      <c r="K44" s="9"/>
-      <c r="L44" s="71" t="s">
-        <v>151</v>
-      </c>
-      <c r="M44" s="72"/>
-      <c r="N44" s="72"/>
-      <c r="O44" s="65">
-        <f>O43/5</f>
+      <c r="O43" s="65">
+        <f>O42/5</f>
         <v>8.4899999999999984</v>
       </c>
-      <c r="P44" s="42"/>
+      <c r="P43" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="J1:P1"/>
     <mergeCell ref="P3:P8"/>
+    <mergeCell ref="L42:N42"/>
     <mergeCell ref="L43:N43"/>
-    <mergeCell ref="L44:N44"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="M12" r:id="rId1"/>

</xml_diff>

<commit_message>
#16 Client BOM Final
</commit_message>
<xml_diff>
--- a/Design Files/LTE-Module-v2.0/BOM/Client_BOM_v2.0.xlsx
+++ b/Design Files/LTE-Module-v2.0/BOM/Client_BOM_v2.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="175">
   <si>
     <t>Component list</t>
   </si>
@@ -438,9 +438,6 @@
     <t>Quantity</t>
   </si>
   <si>
-    <t>Alternate Part Number</t>
-  </si>
-  <si>
     <t>Quantity (5 Boards)</t>
   </si>
   <si>
@@ -459,28 +456,7 @@
     <t xml:space="preserve"> Remarks</t>
   </si>
   <si>
-    <t>Links</t>
-  </si>
-  <si>
-    <t>Digikey</t>
-  </si>
-  <si>
-    <t>Unit Cost (5 Boards)</t>
-  </si>
-  <si>
-    <t>Total Cost (5 Boards)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total Component Cost </t>
-  </si>
-  <si>
-    <t>Single Board Cost</t>
-  </si>
-  <si>
     <t>Peripheral</t>
-  </si>
-  <si>
-    <t>Custom Supplier</t>
   </si>
   <si>
     <t>HJ Tech</t>
@@ -574,12 +550,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="3">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
-    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
-    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -719,14 +693,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="14"/>
       <name val="Calibri"/>
@@ -760,7 +726,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="20">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -968,25 +934,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1140,34 +1092,16 @@
     <xf numFmtId="0" fontId="19" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="17" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="14" fillId="3" borderId="14" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="14" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1177,17 +1111,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1213,13 +1138,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>15</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>47625</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>19942</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>1905000</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>171450</xdr:rowOff>
@@ -1527,7 +1452,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:P43"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="25" customWidth="1"/>
@@ -1537,17 +1462,13 @@
     <col min="6" max="6" width="26.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.5703125" customWidth="1"/>
-    <col min="14" max="14" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="29.42578125" customWidth="1"/>
+    <col min="9" max="9" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="29.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -1556,16 +1477,12 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="68"/>
-      <c r="K1" s="68"/>
-      <c r="L1" s="68"/>
-      <c r="M1" s="68"/>
-      <c r="N1" s="68"/>
-      <c r="O1" s="68"/>
-      <c r="P1" s="68"/>
-    </row>
-    <row r="2" spans="1:16" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="61"/>
+      <c r="L1" s="61"/>
+    </row>
+    <row r="2" spans="1:12" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="20"/>
       <c r="C2" s="43"/>
@@ -1574,20 +1491,16 @@
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="51" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="3"/>
-      <c r="I2" s="11"/>
+      <c r="I2" s="3"/>
       <c r="J2" s="3"/>
       <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
-      <c r="O2" s="3"/>
-      <c r="P2" s="40"/>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="L2" s="40"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="21"/>
       <c r="C3" s="44"/>
@@ -1596,20 +1509,16 @@
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="52" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="4"/>
-      <c r="I3" s="12"/>
+      <c r="I3" s="4"/>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="4"/>
-      <c r="P3" s="69"/>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="L3" s="62"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="21"/>
       <c r="C4" s="44"/>
@@ -1618,20 +1527,16 @@
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="53" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="G4" s="13"/>
       <c r="H4" s="6"/>
-      <c r="I4" s="13"/>
+      <c r="I4" s="6"/>
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
-      <c r="L4" s="6"/>
-      <c r="M4" s="58"/>
-      <c r="N4" s="58"/>
-      <c r="O4" s="58"/>
-      <c r="P4" s="70"/>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="L4" s="63"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="21"/>
       <c r="C5" s="44"/>
@@ -1644,16 +1549,12 @@
       </c>
       <c r="G5" s="14"/>
       <c r="H5" s="5"/>
-      <c r="I5" s="14"/>
+      <c r="I5" s="5"/>
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
-      <c r="L5" s="5"/>
-      <c r="M5" s="58"/>
-      <c r="N5" s="58"/>
-      <c r="O5" s="58"/>
-      <c r="P5" s="70"/>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="L5" s="63"/>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="22"/>
       <c r="C6" s="45"/>
@@ -1662,16 +1563,12 @@
       <c r="F6" s="16"/>
       <c r="G6" s="14"/>
       <c r="H6" s="5"/>
-      <c r="I6" s="14"/>
+      <c r="I6" s="5"/>
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
-      <c r="L6" s="5"/>
-      <c r="M6" s="58"/>
-      <c r="N6" s="58"/>
-      <c r="O6" s="58"/>
-      <c r="P6" s="70"/>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="L6" s="63"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="23"/>
       <c r="C7" s="46"/>
@@ -1680,16 +1577,12 @@
       <c r="F7" s="18"/>
       <c r="G7" s="17"/>
       <c r="H7" s="7"/>
-      <c r="I7" s="17"/>
+      <c r="I7" s="7"/>
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
-      <c r="L7" s="7"/>
-      <c r="M7" s="7"/>
-      <c r="N7" s="7"/>
-      <c r="O7" s="7"/>
-      <c r="P7" s="70"/>
-    </row>
-    <row r="8" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L7" s="63"/>
+    </row>
+    <row r="8" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="26"/>
       <c r="C8" s="47"/>
@@ -1698,16 +1591,12 @@
       <c r="F8" s="28"/>
       <c r="G8" s="17"/>
       <c r="H8" s="7"/>
-      <c r="I8" s="17"/>
+      <c r="I8" s="7"/>
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
-      <c r="L8" s="7"/>
-      <c r="M8" s="7"/>
-      <c r="N8" s="7"/>
-      <c r="O8" s="7"/>
-      <c r="P8" s="70"/>
-    </row>
-    <row r="9" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L8" s="63"/>
+    </row>
+    <row r="9" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="29" t="s">
         <v>4</v>
@@ -1731,80 +1620,55 @@
         <v>110</v>
       </c>
       <c r="I9" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="J9" s="29" t="s">
+        <v>138</v>
+      </c>
+      <c r="K9" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="J9" s="29" t="s">
-        <v>141</v>
-      </c>
-      <c r="K9" s="29" t="s">
-        <v>138</v>
-      </c>
       <c r="L9" s="29" t="s">
-        <v>140</v>
-      </c>
-      <c r="M9" s="29" t="s">
-        <v>146</v>
-      </c>
-      <c r="N9" s="29" t="s">
-        <v>148</v>
-      </c>
-      <c r="O9" s="29" t="s">
-        <v>149</v>
-      </c>
-      <c r="P9" s="29" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="50">
         <f>ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
       <c r="C10" s="56" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="D10" s="36" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="E10" s="36" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="F10" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G10" s="36" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="H10" s="36" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="I10" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J10" s="36" t="s">
-        <v>142</v>
+        <v>141</v>
+      </c>
+      <c r="J10" s="36">
+        <v>1</v>
       </c>
       <c r="K10" s="36">
-        <v>1</v>
-      </c>
-      <c r="L10" s="36">
-        <f>K10*5</f>
+        <f>J10*5</f>
         <v>5</v>
       </c>
-      <c r="M10" s="59" t="s">
-        <v>147</v>
-      </c>
-      <c r="N10" s="61">
-        <v>1.59</v>
-      </c>
-      <c r="O10" s="61">
-        <f>N10*L10</f>
-        <v>7.95</v>
-      </c>
-      <c r="P10" s="36"/>
-    </row>
-    <row r="11" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L10" s="36"/>
+    </row>
+    <row r="11" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="50">
         <f t="shared" ref="B11:B41" si="0">ROW(B11) - ROW($B$9)</f>
@@ -1817,43 +1681,30 @@
         <v>18</v>
       </c>
       <c r="E11" s="38" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="F11" s="38" t="s">
         <v>70</v>
       </c>
       <c r="G11" s="38" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="H11" s="38" t="s">
         <v>112</v>
       </c>
-      <c r="I11" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J11" s="38" t="s">
-        <v>169</v>
+      <c r="I11" s="38" t="s">
+        <v>161</v>
+      </c>
+      <c r="J11" s="38">
+        <v>1</v>
       </c>
       <c r="K11" s="38">
-        <v>1</v>
-      </c>
-      <c r="L11" s="38">
-        <f t="shared" ref="L11" si="1">K11*5</f>
+        <f t="shared" ref="K11" si="1">J11*5</f>
         <v>5</v>
       </c>
-      <c r="M11" s="60" t="s">
-        <v>147</v>
-      </c>
-      <c r="N11" s="62">
-        <v>0.1</v>
-      </c>
-      <c r="O11" s="61">
-        <f t="shared" ref="O11:O29" si="2">N11*L11</f>
-        <v>0.5</v>
-      </c>
-      <c r="P11" s="38"/>
-    </row>
-    <row r="12" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L11" s="38"/>
+    </row>
+    <row r="12" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="50">
         <f>ROW(B12) - ROW($B$9)</f>
@@ -1878,31 +1729,18 @@
         <v>111</v>
       </c>
       <c r="I12" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J12" s="36" t="s">
         <v>126</v>
       </c>
+      <c r="J12" s="36">
+        <v>1</v>
+      </c>
       <c r="K12" s="36">
-        <v>1</v>
-      </c>
-      <c r="L12" s="36">
-        <f>K12*5</f>
+        <f>J12*5</f>
         <v>5</v>
       </c>
-      <c r="M12" s="59" t="s">
-        <v>147</v>
-      </c>
-      <c r="N12" s="61">
-        <v>0.1</v>
-      </c>
-      <c r="O12" s="61">
-        <f t="shared" si="2"/>
-        <v>0.5</v>
-      </c>
-      <c r="P12" s="36"/>
-    </row>
-    <row r="13" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L12" s="36"/>
+    </row>
+    <row r="13" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="50">
         <f t="shared" si="0"/>
@@ -1912,7 +1750,7 @@
         <v>7</v>
       </c>
       <c r="D13" s="38" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="E13" s="39" t="s">
         <v>44</v>
@@ -1926,32 +1764,19 @@
       <c r="H13" s="38" t="s">
         <v>112</v>
       </c>
-      <c r="I13" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J13" s="38" t="s">
+      <c r="I13" s="38" t="s">
         <v>127</v>
       </c>
+      <c r="J13" s="38">
+        <v>6</v>
+      </c>
       <c r="K13" s="38">
-        <v>6</v>
-      </c>
-      <c r="L13" s="38">
-        <f t="shared" ref="L13" si="3">K13*5</f>
+        <f t="shared" ref="K13" si="2">J13*5</f>
         <v>30</v>
       </c>
-      <c r="M13" s="60" t="s">
-        <v>147</v>
-      </c>
-      <c r="N13" s="62">
-        <v>0.1</v>
-      </c>
-      <c r="O13" s="61">
-        <f t="shared" si="2"/>
-        <v>3</v>
-      </c>
-      <c r="P13" s="38"/>
-    </row>
-    <row r="14" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L13" s="38"/>
+    </row>
+    <row r="14" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="50">
         <f>ROW(B14) - ROW($B$9)</f>
@@ -1964,43 +1789,30 @@
         <v>20</v>
       </c>
       <c r="E14" s="36" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="F14" s="36" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="G14" s="36" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="H14" s="36" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="I14" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J14" s="36" t="s">
         <v>128</v>
       </c>
+      <c r="J14" s="36">
+        <v>1</v>
+      </c>
       <c r="K14" s="36">
-        <v>1</v>
-      </c>
-      <c r="L14" s="36">
-        <f>K14*5</f>
+        <f>J14*5</f>
         <v>5</v>
       </c>
-      <c r="M14" s="60" t="s">
-        <v>147</v>
-      </c>
-      <c r="N14" s="61">
-        <v>1.04</v>
-      </c>
-      <c r="O14" s="61">
-        <f t="shared" si="2"/>
-        <v>5.2</v>
-      </c>
-      <c r="P14" s="36"/>
-    </row>
-    <row r="15" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L14" s="36"/>
+    </row>
+    <row r="15" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="50">
         <f t="shared" si="0"/>
@@ -2024,32 +1836,19 @@
       <c r="H15" s="38" t="s">
         <v>112</v>
       </c>
-      <c r="I15" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J15" s="38" t="s">
+      <c r="I15" s="38" t="s">
         <v>129</v>
       </c>
+      <c r="J15" s="38">
+        <v>1</v>
+      </c>
       <c r="K15" s="38">
-        <v>1</v>
-      </c>
-      <c r="L15" s="38">
-        <f t="shared" ref="L15" si="4">K15*5</f>
+        <f t="shared" ref="K15" si="3">J15*5</f>
         <v>5</v>
       </c>
-      <c r="M15" s="60" t="s">
-        <v>147</v>
-      </c>
-      <c r="N15" s="62">
-        <v>0.1</v>
-      </c>
-      <c r="O15" s="61">
-        <f t="shared" si="2"/>
-        <v>0.5</v>
-      </c>
-      <c r="P15" s="38"/>
-    </row>
-    <row r="16" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L15" s="38"/>
+    </row>
+    <row r="16" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="50">
         <f>ROW(B16) - ROW($B$9)</f>
@@ -2074,31 +1873,18 @@
         <v>112</v>
       </c>
       <c r="I16" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J16" s="36" t="s">
         <v>130</v>
       </c>
+      <c r="J16" s="36">
+        <v>3</v>
+      </c>
       <c r="K16" s="36">
-        <v>3</v>
-      </c>
-      <c r="L16" s="36">
-        <f>K16*5</f>
+        <f>J16*5</f>
         <v>15</v>
       </c>
-      <c r="M16" s="59" t="s">
-        <v>147</v>
-      </c>
-      <c r="N16" s="61">
-        <v>0.1</v>
-      </c>
-      <c r="O16" s="61">
-        <f t="shared" si="2"/>
-        <v>1.5</v>
-      </c>
-      <c r="P16" s="36"/>
-    </row>
-    <row r="17" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L16" s="36"/>
+    </row>
+    <row r="17" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="50">
         <f t="shared" si="0"/>
@@ -2122,32 +1908,19 @@
       <c r="H17" s="38" t="s">
         <v>113</v>
       </c>
-      <c r="I17" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J17" s="38" t="s">
+      <c r="I17" s="38" t="s">
         <v>131</v>
       </c>
+      <c r="J17" s="38">
+        <v>2</v>
+      </c>
       <c r="K17" s="38">
-        <v>2</v>
-      </c>
-      <c r="L17" s="38">
-        <f t="shared" ref="L17" si="5">K17*5</f>
+        <f t="shared" ref="K17" si="4">J17*5</f>
         <v>10</v>
       </c>
-      <c r="M17" s="59" t="s">
-        <v>147</v>
-      </c>
-      <c r="N17" s="62">
-        <v>0.11</v>
-      </c>
-      <c r="O17" s="61">
-        <f t="shared" si="2"/>
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="P17" s="38"/>
-    </row>
-    <row r="18" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L17" s="38"/>
+    </row>
+    <row r="18" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="50">
         <f>ROW(B18) - ROW($B$9)</f>
@@ -2172,31 +1945,18 @@
         <v>114</v>
       </c>
       <c r="I18" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J18" s="36" t="s">
-        <v>142</v>
+        <v>141</v>
+      </c>
+      <c r="J18" s="36">
+        <v>1</v>
       </c>
       <c r="K18" s="36">
-        <v>1</v>
-      </c>
-      <c r="L18" s="36">
-        <f>K18*5</f>
+        <f>J18*5</f>
         <v>5</v>
       </c>
-      <c r="M18" s="59" t="s">
-        <v>147</v>
-      </c>
-      <c r="N18" s="61">
-        <v>0.23</v>
-      </c>
-      <c r="O18" s="61">
-        <f t="shared" si="2"/>
-        <v>1.1500000000000001</v>
-      </c>
-      <c r="P18" s="36"/>
-    </row>
-    <row r="19" spans="1:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L18" s="36"/>
+    </row>
+    <row r="19" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="50">
         <f t="shared" si="0"/>
@@ -2220,30 +1980,19 @@
       <c r="H19" s="38" t="s">
         <v>115</v>
       </c>
-      <c r="I19" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J19" s="38" t="s">
-        <v>142</v>
+      <c r="I19" s="38" t="s">
+        <v>141</v>
+      </c>
+      <c r="J19" s="38">
+        <v>2</v>
       </c>
       <c r="K19" s="38">
-        <v>2</v>
-      </c>
-      <c r="L19" s="38">
-        <f t="shared" ref="L19" si="6">K19*5</f>
+        <f t="shared" ref="K19" si="5">J19*5</f>
         <v>10</v>
       </c>
-      <c r="M19" s="60" t="s">
-        <v>153</v>
-      </c>
-      <c r="N19" s="62"/>
-      <c r="O19" s="61">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="P19" s="38"/>
-    </row>
-    <row r="20" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L19" s="38"/>
+    </row>
+    <row r="20" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="50">
         <f>ROW(B20) - ROW($B$9)</f>
@@ -2268,31 +2017,18 @@
         <v>116</v>
       </c>
       <c r="I20" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J20" s="36" t="s">
-        <v>142</v>
+        <v>141</v>
+      </c>
+      <c r="J20" s="36">
+        <v>1</v>
       </c>
       <c r="K20" s="36">
-        <v>1</v>
-      </c>
-      <c r="L20" s="36">
-        <f>K20*5</f>
+        <f>J20*5</f>
         <v>5</v>
       </c>
-      <c r="M20" s="59" t="s">
-        <v>147</v>
-      </c>
-      <c r="N20" s="61">
-        <v>0.48</v>
-      </c>
-      <c r="O20" s="61">
-        <f t="shared" si="2"/>
-        <v>2.4</v>
-      </c>
-      <c r="P20" s="36"/>
-    </row>
-    <row r="21" spans="1:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L20" s="36"/>
+    </row>
+    <row r="21" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="50">
         <f t="shared" si="0"/>
@@ -2316,30 +2052,19 @@
       <c r="H21" s="38" t="s">
         <v>117</v>
       </c>
-      <c r="I21" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J21" s="38" t="s">
-        <v>142</v>
+      <c r="I21" s="38" t="s">
+        <v>141</v>
+      </c>
+      <c r="J21" s="38">
+        <v>1</v>
       </c>
       <c r="K21" s="38">
-        <v>1</v>
-      </c>
-      <c r="L21" s="38">
-        <f t="shared" ref="L21" si="7">K21*5</f>
+        <f t="shared" ref="K21" si="6">J21*5</f>
         <v>5</v>
       </c>
-      <c r="M21" s="60" t="s">
-        <v>153</v>
-      </c>
-      <c r="N21" s="62"/>
-      <c r="O21" s="61">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="P21" s="38"/>
-    </row>
-    <row r="22" spans="1:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L21" s="38"/>
+    </row>
+    <row r="22" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="50">
         <f>ROW(B22) - ROW($B$9)</f>
@@ -2364,83 +2089,61 @@
         <v>118</v>
       </c>
       <c r="I22" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J22" s="36" t="s">
-        <v>142</v>
+        <v>141</v>
+      </c>
+      <c r="J22" s="36">
+        <v>1</v>
       </c>
       <c r="K22" s="36">
-        <v>1</v>
-      </c>
-      <c r="L22" s="36">
-        <f>K22*5</f>
+        <f>J22*5</f>
         <v>5</v>
       </c>
-      <c r="M22" s="60" t="s">
-        <v>153</v>
-      </c>
-      <c r="N22" s="61"/>
-      <c r="O22" s="61">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="P22" s="36"/>
-    </row>
-    <row r="23" spans="1:16" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L22" s="36"/>
+    </row>
+    <row r="23" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="50">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="C23" s="57" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="D23" s="38" t="s">
         <v>29</v>
       </c>
       <c r="E23" s="38" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="F23" s="38" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G23" s="38" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="H23" s="38" t="s">
-        <v>154</v>
-      </c>
-      <c r="I23" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J23" s="38" t="s">
-        <v>142</v>
+        <v>146</v>
+      </c>
+      <c r="I23" s="38" t="s">
+        <v>141</v>
+      </c>
+      <c r="J23" s="38">
+        <v>1</v>
       </c>
       <c r="K23" s="38">
-        <v>1</v>
-      </c>
-      <c r="L23" s="38">
-        <f t="shared" ref="L23" si="8">K23*5</f>
+        <f t="shared" ref="K23" si="7">J23*5</f>
         <v>5</v>
       </c>
-      <c r="M23" s="60" t="s">
-        <v>153</v>
-      </c>
-      <c r="N23" s="62"/>
-      <c r="O23" s="61">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="P23" s="38"/>
-    </row>
-    <row r="24" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L23" s="38"/>
+    </row>
+    <row r="24" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="50">
         <f>ROW(B24) - ROW($B$9)</f>
         <v>15</v>
       </c>
       <c r="C24" s="56" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D24" s="36" t="s">
         <v>30</v>
@@ -2449,38 +2152,27 @@
         <v>53</v>
       </c>
       <c r="F24" s="55" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G24" s="37" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H24" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="I24" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J24" s="55" t="s">
-        <v>142</v>
+        <v>141</v>
+      </c>
+      <c r="I24" s="55" t="s">
+        <v>141</v>
+      </c>
+      <c r="J24" s="36">
+        <v>1</v>
       </c>
       <c r="K24" s="36">
-        <v>1</v>
-      </c>
-      <c r="L24" s="36">
-        <f>K24*5</f>
+        <f>J24*5</f>
         <v>5</v>
       </c>
-      <c r="M24" s="55" t="s">
-        <v>142</v>
-      </c>
-      <c r="N24" s="61"/>
-      <c r="O24" s="61">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="P24" s="36"/>
-    </row>
-    <row r="25" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L24" s="36"/>
+    </row>
+    <row r="25" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="50">
         <f t="shared" si="0"/>
@@ -2496,38 +2188,27 @@
         <v>54</v>
       </c>
       <c r="F25" s="38" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G25" s="39" t="s">
         <v>97</v>
       </c>
       <c r="H25" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="I25" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J25" s="55" t="s">
-        <v>142</v>
+        <v>141</v>
+      </c>
+      <c r="I25" s="55" t="s">
+        <v>141</v>
+      </c>
+      <c r="J25" s="38">
+        <v>1</v>
       </c>
       <c r="K25" s="38">
-        <v>1</v>
-      </c>
-      <c r="L25" s="38">
-        <f t="shared" ref="L25" si="9">K25*5</f>
+        <f t="shared" ref="K25" si="8">J25*5</f>
         <v>5</v>
       </c>
-      <c r="M25" s="55" t="s">
-        <v>142</v>
-      </c>
-      <c r="N25" s="62"/>
-      <c r="O25" s="61">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="P25" s="38"/>
-    </row>
-    <row r="26" spans="1:16" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L25" s="38"/>
+    </row>
+    <row r="26" spans="1:12" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="50">
         <f>ROW(B26) - ROW($B$9)</f>
@@ -2537,13 +2218,13 @@
         <v>11</v>
       </c>
       <c r="D26" s="36" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E26" s="37" t="s">
         <v>55</v>
       </c>
       <c r="F26" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G26" s="37" t="s">
         <v>78</v>
@@ -2552,29 +2233,18 @@
         <v>119</v>
       </c>
       <c r="I26" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J26" s="36" t="s">
-        <v>142</v>
+        <v>141</v>
+      </c>
+      <c r="J26" s="36">
+        <v>2</v>
       </c>
       <c r="K26" s="36">
-        <v>2</v>
-      </c>
-      <c r="L26" s="36">
-        <f>K26*5</f>
+        <f>J26*5</f>
         <v>10</v>
       </c>
-      <c r="M26" s="60" t="s">
-        <v>153</v>
-      </c>
-      <c r="N26" s="61"/>
-      <c r="O26" s="61">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="P26" s="36"/>
-    </row>
-    <row r="27" spans="1:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L26" s="36"/>
+    </row>
+    <row r="27" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="50">
         <f>ROW(B27) - ROW($B$9)</f>
@@ -2599,29 +2269,18 @@
         <v>120</v>
       </c>
       <c r="I27" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J27" s="36" t="s">
-        <v>142</v>
+        <v>141</v>
+      </c>
+      <c r="J27" s="36">
+        <v>1</v>
       </c>
       <c r="K27" s="36">
-        <v>1</v>
-      </c>
-      <c r="L27" s="36">
-        <f>K27*5</f>
+        <f>J27*5</f>
         <v>5</v>
       </c>
-      <c r="M27" s="60" t="s">
-        <v>153</v>
-      </c>
-      <c r="N27" s="61"/>
-      <c r="O27" s="61">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="P27" s="36"/>
-    </row>
-    <row r="28" spans="1:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L27" s="36"/>
+    </row>
+    <row r="28" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="50">
         <f t="shared" si="0"/>
@@ -2645,30 +2304,19 @@
       <c r="H28" s="38" t="s">
         <v>120</v>
       </c>
-      <c r="I28" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J28" s="38" t="s">
-        <v>142</v>
+      <c r="I28" s="38" t="s">
+        <v>141</v>
+      </c>
+      <c r="J28" s="38">
+        <v>1</v>
       </c>
       <c r="K28" s="38">
-        <v>1</v>
-      </c>
-      <c r="L28" s="38">
-        <f t="shared" ref="L28" si="10">K28*5</f>
+        <f t="shared" ref="K28" si="9">J28*5</f>
         <v>5</v>
       </c>
-      <c r="M28" s="60" t="s">
-        <v>153</v>
-      </c>
-      <c r="N28" s="62"/>
-      <c r="O28" s="61">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="P28" s="38"/>
-    </row>
-    <row r="29" spans="1:16" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L28" s="38"/>
+    </row>
+    <row r="29" spans="1:12" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="50">
         <f>ROW(B29) - ROW($B$9)</f>
@@ -2693,29 +2341,18 @@
         <v>121</v>
       </c>
       <c r="I29" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J29" s="36" t="s">
-        <v>142</v>
+        <v>141</v>
+      </c>
+      <c r="J29" s="36">
+        <v>4</v>
       </c>
       <c r="K29" s="36">
-        <v>4</v>
-      </c>
-      <c r="L29" s="36">
-        <f>K29*5</f>
+        <f>J29*5</f>
         <v>20</v>
       </c>
-      <c r="M29" s="60" t="s">
-        <v>153</v>
-      </c>
-      <c r="N29" s="61"/>
-      <c r="O29" s="61">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="P29" s="36"/>
-    </row>
-    <row r="30" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L29" s="36"/>
+    </row>
+    <row r="30" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="50">
         <f>ROW(B30) - ROW($B$9)</f>
@@ -2725,7 +2362,7 @@
         <v>14</v>
       </c>
       <c r="D30" s="36" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="E30" s="37" t="s">
         <v>64</v>
@@ -2740,31 +2377,18 @@
         <v>112</v>
       </c>
       <c r="I30" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J30" s="36" t="s">
         <v>137</v>
       </c>
+      <c r="J30" s="36">
+        <v>3</v>
+      </c>
       <c r="K30" s="36">
-        <v>3</v>
-      </c>
-      <c r="L30" s="36">
-        <f>K30*5</f>
+        <f>J30*5</f>
         <v>15</v>
       </c>
-      <c r="M30" s="59" t="s">
-        <v>147</v>
-      </c>
-      <c r="N30" s="62">
-        <v>0.1</v>
-      </c>
-      <c r="O30" s="63">
-        <f>N30*L30</f>
-        <v>1.5</v>
-      </c>
-      <c r="P30" s="36"/>
-    </row>
-    <row r="31" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L30" s="36"/>
+    </row>
+    <row r="31" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="50">
         <f>ROW(B31) - ROW($B$9)</f>
@@ -2789,31 +2413,18 @@
         <v>112</v>
       </c>
       <c r="I31" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J31" s="36" t="s">
         <v>133</v>
       </c>
+      <c r="J31" s="36">
+        <v>2</v>
+      </c>
       <c r="K31" s="36">
-        <v>2</v>
-      </c>
-      <c r="L31" s="36">
-        <f>K31*5</f>
+        <f>J31*5</f>
         <v>10</v>
       </c>
-      <c r="M31" s="59" t="s">
-        <v>147</v>
-      </c>
-      <c r="N31" s="62">
-        <v>0.1</v>
-      </c>
-      <c r="O31" s="63">
-        <f>N31*L31</f>
-        <v>1</v>
-      </c>
-      <c r="P31" s="36"/>
-    </row>
-    <row r="32" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L31" s="36"/>
+    </row>
+    <row r="32" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="50">
         <f t="shared" si="0"/>
@@ -2823,7 +2434,7 @@
         <v>14</v>
       </c>
       <c r="D32" s="36" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="E32" s="39" t="s">
         <v>59</v>
@@ -2837,32 +2448,19 @@
       <c r="H32" s="38" t="s">
         <v>112</v>
       </c>
-      <c r="I32" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J32" s="38" t="s">
+      <c r="I32" s="38" t="s">
         <v>132</v>
       </c>
+      <c r="J32" s="38">
+        <v>2</v>
+      </c>
       <c r="K32" s="38">
-        <v>2</v>
-      </c>
-      <c r="L32" s="38">
-        <f t="shared" ref="L32" si="11">K32*5</f>
+        <f t="shared" ref="K32" si="10">J32*5</f>
         <v>10</v>
       </c>
-      <c r="M32" s="59" t="s">
-        <v>147</v>
-      </c>
-      <c r="N32" s="62">
-        <v>0.1</v>
-      </c>
-      <c r="O32" s="63">
-        <f>N32*L32</f>
-        <v>1</v>
-      </c>
-      <c r="P32" s="38"/>
-    </row>
-    <row r="33" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L32" s="38"/>
+    </row>
+    <row r="33" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="50">
         <f t="shared" si="0"/>
@@ -2886,32 +2484,19 @@
       <c r="H33" s="38" t="s">
         <v>112</v>
       </c>
-      <c r="I33" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J33" s="38" t="s">
+      <c r="I33" s="38" t="s">
         <v>134</v>
       </c>
+      <c r="J33" s="38">
+        <v>2</v>
+      </c>
       <c r="K33" s="38">
-        <v>2</v>
-      </c>
-      <c r="L33" s="38">
-        <f t="shared" ref="L33" si="12">K33*5</f>
+        <f t="shared" ref="K33" si="11">J33*5</f>
         <v>10</v>
       </c>
-      <c r="M33" s="59" t="s">
-        <v>147</v>
-      </c>
-      <c r="N33" s="62">
-        <v>0.1</v>
-      </c>
-      <c r="O33" s="63">
-        <f t="shared" ref="O33:O39" si="13">N33*L33</f>
-        <v>1</v>
-      </c>
-      <c r="P33" s="38"/>
-    </row>
-    <row r="34" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L33" s="38"/>
+    </row>
+    <row r="34" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="50">
         <f>ROW(B34) - ROW($B$9)</f>
@@ -2936,31 +2521,18 @@
         <v>112</v>
       </c>
       <c r="I34" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J34" s="36" t="s">
         <v>135</v>
       </c>
+      <c r="J34" s="36">
+        <v>4</v>
+      </c>
       <c r="K34" s="36">
-        <v>4</v>
-      </c>
-      <c r="L34" s="36">
-        <f>K34*5</f>
+        <f>J34*5</f>
         <v>20</v>
       </c>
-      <c r="M34" s="59" t="s">
-        <v>147</v>
-      </c>
-      <c r="N34" s="62">
-        <v>0.1</v>
-      </c>
-      <c r="O34" s="63">
-        <f t="shared" si="13"/>
-        <v>2</v>
-      </c>
-      <c r="P34" s="36"/>
-    </row>
-    <row r="35" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L34" s="36"/>
+    </row>
+    <row r="35" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="50">
         <f t="shared" si="0"/>
@@ -2984,32 +2556,19 @@
       <c r="H35" s="38" t="s">
         <v>112</v>
       </c>
-      <c r="I35" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J35" s="38" t="s">
+      <c r="I35" s="38" t="s">
         <v>136</v>
       </c>
+      <c r="J35" s="38">
+        <v>4</v>
+      </c>
       <c r="K35" s="38">
-        <v>4</v>
-      </c>
-      <c r="L35" s="38">
-        <f t="shared" ref="L35" si="14">K35*5</f>
+        <f t="shared" ref="K35" si="12">J35*5</f>
         <v>20</v>
       </c>
-      <c r="M35" s="59" t="s">
-        <v>147</v>
-      </c>
-      <c r="N35" s="62">
-        <v>0.1</v>
-      </c>
-      <c r="O35" s="63">
-        <f t="shared" si="13"/>
-        <v>2</v>
-      </c>
-      <c r="P35" s="38"/>
-    </row>
-    <row r="36" spans="1:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L35" s="38"/>
+    </row>
+    <row r="36" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="B36" s="50">
         <f t="shared" si="0"/>
@@ -3025,7 +2584,7 @@
         <v>65</v>
       </c>
       <c r="F36" s="38" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G36" s="39" t="s">
         <v>82</v>
@@ -3033,30 +2592,19 @@
       <c r="H36" s="38" t="s">
         <v>122</v>
       </c>
-      <c r="I36" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J36" s="38" t="s">
-        <v>142</v>
+      <c r="I36" s="38" t="s">
+        <v>141</v>
+      </c>
+      <c r="J36" s="38">
+        <v>1</v>
       </c>
       <c r="K36" s="38">
-        <v>1</v>
-      </c>
-      <c r="L36" s="38">
-        <f t="shared" ref="L36" si="15">K36*5</f>
+        <f t="shared" ref="K36" si="13">J36*5</f>
         <v>5</v>
       </c>
-      <c r="M36" s="60" t="s">
-        <v>153</v>
-      </c>
-      <c r="N36" s="62"/>
-      <c r="O36" s="63">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="P36" s="38"/>
-    </row>
-    <row r="37" spans="1:16" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L36" s="38"/>
+    </row>
+    <row r="37" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" s="50">
         <f>ROW(B37) - ROW($B$9)</f>
@@ -3081,31 +2629,18 @@
         <v>123</v>
       </c>
       <c r="I37" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J37" s="36" t="s">
-        <v>142</v>
+        <v>141</v>
+      </c>
+      <c r="J37" s="36">
+        <v>1</v>
       </c>
       <c r="K37" s="36">
-        <v>1</v>
-      </c>
-      <c r="L37" s="36">
-        <f>K37*5</f>
+        <f>J37*5</f>
         <v>5</v>
       </c>
-      <c r="M37" s="59" t="s">
-        <v>147</v>
-      </c>
-      <c r="N37" s="61">
-        <v>0.95</v>
-      </c>
-      <c r="O37" s="63">
-        <f t="shared" si="13"/>
-        <v>4.75</v>
-      </c>
-      <c r="P37" s="36"/>
-    </row>
-    <row r="38" spans="1:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L37" s="36"/>
+    </row>
+    <row r="38" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
       <c r="B38" s="50">
         <f>ROW(B38) - ROW($B$9)</f>
@@ -3115,7 +2650,7 @@
         <v>16</v>
       </c>
       <c r="D38" s="36" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="E38" s="37" t="s">
         <v>67</v>
@@ -3130,29 +2665,18 @@
         <v>124</v>
       </c>
       <c r="I38" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J38" s="36" t="s">
-        <v>142</v>
+        <v>141</v>
+      </c>
+      <c r="J38" s="36">
+        <v>1</v>
       </c>
       <c r="K38" s="36">
-        <v>1</v>
-      </c>
-      <c r="L38" s="36">
-        <f>K38*5</f>
+        <f>J38*5</f>
         <v>5</v>
       </c>
-      <c r="M38" s="60" t="s">
-        <v>153</v>
-      </c>
-      <c r="N38" s="61"/>
-      <c r="O38" s="63">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="P38" s="36"/>
-    </row>
-    <row r="39" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L38" s="36"/>
+    </row>
+    <row r="39" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
       <c r="B39" s="50">
         <f t="shared" si="0"/>
@@ -3176,124 +2700,89 @@
       <c r="H39" s="38" t="s">
         <v>125</v>
       </c>
-      <c r="I39" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J39" s="38" t="s">
-        <v>142</v>
+      <c r="I39" s="38" t="s">
+        <v>141</v>
+      </c>
+      <c r="J39" s="38">
+        <v>1</v>
       </c>
       <c r="K39" s="38">
-        <v>1</v>
-      </c>
-      <c r="L39" s="38">
-        <f t="shared" ref="L39:L41" si="16">K39*5</f>
+        <f t="shared" ref="K39:K41" si="14">J39*5</f>
         <v>5</v>
       </c>
-      <c r="M39" s="59" t="s">
-        <v>147</v>
-      </c>
-      <c r="N39" s="62">
-        <v>1.08</v>
-      </c>
-      <c r="O39" s="63">
-        <f t="shared" si="13"/>
-        <v>5.4</v>
-      </c>
-      <c r="P39" s="38"/>
-    </row>
-    <row r="40" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+      <c r="L39" s="38"/>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
-      <c r="B40" s="66">
+      <c r="B40" s="58">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
       <c r="C40" s="57" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="D40" s="38" t="s">
-        <v>142</v>
-      </c>
-      <c r="E40" s="67" t="s">
-        <v>174</v>
-      </c>
-      <c r="F40" s="67"/>
-      <c r="G40" s="67" t="s">
-        <v>175</v>
-      </c>
-      <c r="H40" s="67" t="s">
-        <v>176</v>
-      </c>
-      <c r="I40" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J40" s="38" t="s">
-        <v>142</v>
+        <v>141</v>
+      </c>
+      <c r="E40" s="59" t="s">
+        <v>166</v>
+      </c>
+      <c r="F40" s="59"/>
+      <c r="G40" s="59" t="s">
+        <v>167</v>
+      </c>
+      <c r="H40" s="59" t="s">
+        <v>168</v>
+      </c>
+      <c r="I40" s="38" t="s">
+        <v>141</v>
+      </c>
+      <c r="J40" s="38">
+        <v>1</v>
       </c>
       <c r="K40" s="38">
-        <v>1</v>
-      </c>
-      <c r="L40" s="38">
-        <f t="shared" si="16"/>
+        <f t="shared" si="14"/>
         <v>5</v>
       </c>
-      <c r="M40" s="60" t="s">
-        <v>153</v>
-      </c>
-      <c r="N40" s="61"/>
-      <c r="O40" s="63">
-        <f t="shared" ref="O40" si="17">N40*L40</f>
-        <v>0</v>
-      </c>
-      <c r="P40" s="38"/>
-    </row>
-    <row r="41" spans="1:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L40" s="38"/>
+    </row>
+    <row r="41" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
-      <c r="B41" s="66">
+      <c r="B41" s="58">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="C41" s="57" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="D41" s="38" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E41" s="38" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="F41" s="38" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G41" s="38" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="H41" s="38" t="s">
-        <v>179</v>
-      </c>
-      <c r="I41" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="J41" s="38" t="s">
-        <v>142</v>
+        <v>171</v>
+      </c>
+      <c r="I41" s="38" t="s">
+        <v>141</v>
+      </c>
+      <c r="J41" s="38">
+        <v>1</v>
       </c>
       <c r="K41" s="38">
-        <v>1</v>
-      </c>
-      <c r="L41" s="38">
-        <f t="shared" si="16"/>
+        <f t="shared" si="14"/>
         <v>5</v>
       </c>
-      <c r="M41" s="60" t="s">
-        <v>153</v>
-      </c>
-      <c r="N41" s="61"/>
-      <c r="O41" s="63">
-        <f t="shared" ref="O41" si="18">N41*L41</f>
-        <v>0</v>
-      </c>
-      <c r="P41" s="38"/>
-    </row>
-    <row r="42" spans="1:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L41" s="38"/>
+    </row>
+    <row r="42" spans="1:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
       <c r="B42" s="31"/>
       <c r="C42" s="48"/>
@@ -3304,19 +2793,10 @@
       <c r="H42" s="34"/>
       <c r="I42" s="35"/>
       <c r="J42" s="35"/>
-      <c r="K42" s="35"/>
-      <c r="L42" s="71" t="s">
-        <v>150</v>
-      </c>
-      <c r="M42" s="72"/>
-      <c r="N42" s="72"/>
-      <c r="O42" s="64">
-        <f>SUM(O10:O41)</f>
-        <v>42.449999999999996</v>
-      </c>
-      <c r="P42" s="41"/>
-    </row>
-    <row r="43" spans="1:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K42" s="60"/>
+      <c r="L42" s="41"/>
+    </row>
+    <row r="43" spans="1:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
       <c r="B43" s="24"/>
       <c r="C43" s="49"/>
@@ -3327,47 +2807,16 @@
       <c r="H43" s="9"/>
       <c r="I43" s="9"/>
       <c r="J43" s="9"/>
-      <c r="K43" s="9"/>
-      <c r="L43" s="71" t="s">
-        <v>151</v>
-      </c>
-      <c r="M43" s="72"/>
-      <c r="N43" s="72"/>
-      <c r="O43" s="65">
-        <f>O42/5</f>
-        <v>8.4899999999999984</v>
-      </c>
-      <c r="P43" s="42"/>
+      <c r="K43" s="60"/>
+      <c r="L43" s="42"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="J1:P1"/>
-    <mergeCell ref="P3:P8"/>
-    <mergeCell ref="L42:N42"/>
-    <mergeCell ref="L43:N43"/>
+  <mergeCells count="2">
+    <mergeCell ref="I1:L1"/>
+    <mergeCell ref="L3:L8"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink ref="M12" r:id="rId1"/>
-    <hyperlink ref="M13" r:id="rId2"/>
-    <hyperlink ref="M15" r:id="rId3"/>
-    <hyperlink ref="M16" r:id="rId4"/>
-    <hyperlink ref="M17" r:id="rId5"/>
-    <hyperlink ref="M18" r:id="rId6"/>
-    <hyperlink ref="M20" r:id="rId7"/>
-    <hyperlink ref="M32" r:id="rId8"/>
-    <hyperlink ref="M31" r:id="rId9"/>
-    <hyperlink ref="M33" r:id="rId10"/>
-    <hyperlink ref="M34" r:id="rId11"/>
-    <hyperlink ref="M35" r:id="rId12"/>
-    <hyperlink ref="M30" r:id="rId13"/>
-    <hyperlink ref="M37" r:id="rId14"/>
-    <hyperlink ref="M39" r:id="rId15"/>
-    <hyperlink ref="M14" r:id="rId16"/>
-    <hyperlink ref="M10" r:id="rId17"/>
-    <hyperlink ref="M11" r:id="rId18"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId19"/>
-  <drawing r:id="rId20"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>